<commit_message>
feat: update to english
</commit_message>
<xml_diff>
--- a/notebooks/01_first_analysis/clean.xlsx
+++ b/notebooks/01_first_analysis/clean.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -554,7 +554,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Permiso para usar mis fotos y vídeos Mis datos personales: Nombre y apellidos: Número de DNI o Pasaporte: Correo electrónico: Doy permiso a la Universidad Politécnica de Madrid. La Universidad se llama UPM. Doy permiso para usar mis fotos. Doy permiso para usar mis vídeos. El título es: Todas las opiniones cuentan. La UPM usará las fotos para un proyecto. El proyecto se llama Inclusens 2.0. La UPM usará las fotos en internet. La UPM usará los vídeos en internet. La UPM no ganará dinero con ellos. La UPM pondrá mi nombre en los vídeos. La UPM pondrá mi nombre en las fotos. La UPM usará su canal de Youtube. La UPM usará sus páginas web. La UPM usará redes sociales como X y LinkedIn. Doy permiso para todos los países. Doy permiso para siempre. Mis fotos cumplen las leyes. Mis vídeos cumplen las leyes. La UPM guarda mis datos personales. La UPM usa mis datos para este permiso. La UPM guarda mis datos siempre. Puedo pedir que borren mis datos. Tengo derechos sobre mis datos. Puedo ver mis datos. Puedo cambiar mis datos. Puedo escribir a este correo: oficina-aps@upm.es. También puedo escribir a: proteccion.datos@upm.es. La UPM está en la calle Ramiro de Maeztu 7. El teléfono es 9106 70390. Si hay problemas, puedo avisar a la Agencia de Protección de Datos. Fecha: Firma:</t>
+          <t>Permiso para usar fotos y vídeos Tus datos Nombre y apellidos: Número de DNI o Pasaporte: Correo electrónico: Qué autorizas Das permiso a la Universidad Politécnica de Madrid para usar tus fotos o tus vídeos. La Universidad también se llama UPM. UPM Es el nombre corto de la Universidad Politécnica de Madrid. Tus fotos y vídeos se usan para el proyecto llamado: Con Inclusens todas las opiniones cuentan. Este proyecto crea herramientas para ayudar a personas con dificultades para comprender. Dónde se verán tus fotos y vídeos La Universidad puede publicar las imágenes en estos sitios: En el canal de Youtube de la Universidad. En las páginas de internet de la Universidad sobre aprendizaje e innovación. En la red social X. En la red social Linkedin. Reglas de este permiso La Universidad pondrá tu nombre para decir que tú eres el autor. La Universidad puede usar el vídeo entero o solo una parte. Nadie ganará dinero con tus fotos o vídeos. Tú aseguras que las fotos y vídeos cumplen las leyes. Este permiso es para siempre y para todos los países. Tus derechos y tus datos Tus datos personales son necesarios para gestionar este permiso. Datos personales Es la información que sirve para saber quién eres. Por ejemplo, tu nombre, tu número de DNI o tu correo electrónico. Tus derechos son: Saber qué datos tiene la Universidad sobre ti. Cambiar tus datos si están mal. Pedir que borren tus datos. Pedir que dejen de usar tus datos. Si quieres usar estos derechos, escribe un correo a: proteccion.datos@upm.es Si no estás de acuerdo con cómo usan tus datos, puedes quejarte en la Agencia Española de Protección de Datos. Firma Tú das tu permiso cuando firmas este papel. Fecha: de de 20 Firma: Información sobre la protección de tus datos ¿Quién cuida tus datos? La Universidad Politécnica de Madrid cuida tus datos. Dirección: Calle Ramiro de Maeztu, número 7. Madrid. Teléfono: 91 06 70 390. Correo electrónico: oficina-aps@upm.es ¿Para qué usa la Universidad tus datos? La Universidad usa tus datos para organizar el permiso que has firmado. ¿Cuánto tiempo guarda la Universidad tus datos? La Universidad guarda tus datos siempre, a menos que tú pidas que los borren. ¿Por qué puede la Universidad usar tus datos? La Universidad usa tus datos porque tú has dado tu permiso al firmar. También los usa para cumplir el acuerdo sobre tus fotos y vídeos. ¿Es obligatorio dar tus datos? Sí. Si no das tus datos, la Universidad no puede usar tus fotos o vídeos. ¿Quién más verá tus datos? Cualquier persona que vea los vídeos o fotos podrá ver tu nombre y apellidos. Tú puedes decir que no quieres que aparezca tu nombre.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -569,21 +569,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (Gemini 3.1 Pro)
-Muy A2</t>
+          <t>Gemini 3.1 Pro</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (Gemini 3.1 Pro)
-Muy A2</t>
+          <t>Gemini 3.1 Pro</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AUTORIZACIÓN PARA USAR IMÁGENES Y VÍDEOS Datos personales Nombre y apellidos: Número de DNI o Pasaporte: Correo electrónico: Yo doy permiso a la Universidad Politécnica de Madrid (UPM). La UPM puede usar mis fotos o vídeos del proyecto INCLUSENS 2.0. El título del trabajo es: Todas las opiniones cuentan. Este proyecto ayuda a personas con dificultades para comprender (discapacidad cognitiva). La UPM publicará estos vídeos en internet. Usará su canal de Youtube y sus páginas de educación. También usará las redes sociales X y LinkedIn. La UPM no ganará dinero con estas imágenes. La UPM pondrá mi nombre como autor en los vídeos. Puede usar el vídeo entero o solo una parte. Yo aseguro que mis imágenes cumplen las leyes de protección de datos. Este permiso es para siempre y para todos los países. La UPM es la responsable de cuidar mis datos personales. Usará mis datos solo para gestionar este permiso. Guardará mi información hasta que yo pida borrarla. Debo dar mis datos para que la UPM pueda usar los vídeos. Tengo derecho a ver mis datos y a corregirlos si están mal. También puedo pedir que borren mi información. Puedo escribir un correo a oficina-aps@upm.es para pedir estos cambios. Si no estoy de acuerdo, puedo reclamar en la Agencia Española de Protección de Datos. Fecha: Firma:</t>
+          <t>Autorización para difundir imagen o vídeo Yo, D./Dña. con DNI o pasaporte número y con correo electrónico doy permiso a la Universidad Politécnica de Madrid, UPM, con CIF Q-2818015-F, para difundir imágenes o una grabación en la que participo o que he creado. Título del material Con Inclusens todas las opiniones cuentan Proyecto Aprendizaje-Servicio. Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores. INCLUSENS 2.0. Dónde puede difundir la UPM este material La UPM puede difundir este material en internet. La UPM puede usar estos canales: el canal oficial de YouTube de la UPM el portal de ApS-UPM: https://aprendizajeservicio.upm.es/ el portal de innovación educativa: https://innovacioneducativa.upm.es la red social X: @IEducativa_UPM LinkedIn: www.linkedin.com/in/aps.upm La UPM usa este material solo para la finalidad de este proyecto. La UPM no usa este material con fines comerciales. Condiciones de esta autorización La UPM reconoce de forma expresa tu autoría en el vídeo o en las imágenes. La UPM puede reproducir, distribuir y comunicar la grabación o las imágenes. Puede hacerlo de forma completa o en parte. Puede hacerlo también en internet. La UPM no obtiene beneficio comercial con esta difusión. Tú declaras que el contenido cumple la ley sobre protección de datos personales, derecho a la imagen y propiedad intelectual o industrial. Tú aceptas que, si otra persona presenta una reclamación por estos temas, la UPM no tendrá responsabilidad. Esta autorización no es exclusiva. Esto significa que tú puedes autorizar también a otras personas o entidades. Esta autorización no tiene fecha de fin. Esta autorización vale para cualquier lugar. Fecha y firma Fecha: Firma: Consentimiento para usar tus datos personales He recibido información sobre el uso de mis datos personales. Doy mi consentimiento para que la Universidad Politécnica de Madrid, a través de la Oficina de Aprendizaje Servicio, ApS, use mis datos personales para gestionar todo lo relacionado con esta autorización. Información sobre protección de datos Datos personales Son los datos que sirven para identificarte. Ejemplo: tu nombre, tu DNI o tu correo electrónico. Tratamiento de datos Es el uso de tus datos para una finalidad concreta. Ejemplo: usar tu correo para gestionar esta autorización. Quién usa tus datos La Universidad Politécnica de Madrid. Oficina de Aprendizaje Servicio, ApS. Dirección: Calle Ramiro de Maeztu, 7. 28040 Madrid. Teléfono: 910670390. Correo electrónico: oficina-aps@upm.es Contacto sobre protección de datos Delegado de Protección de Datos Es la persona o el servicio que te ayuda con dudas o problemas sobre el uso de tus datos. Correo electrónico: proteccion.datos@upm.es Para qué usa la UPM tus datos La UPM usa tus datos para gestionar todo lo relacionado con esta autorización. Durante cuánto tiempo guarda la UPM tus datos La UPM guarda tus datos sin fecha de fin. La UPM los guarda hasta que tú pidas su supresión. Por qué la UPM puede usar tus datos La UPM puede usar tus datos por 2 motivos: porque este tratamiento es necesario para gestionar esta autorización porque tú das tu consentimiento para usar tus datos con esta finalidad Si no facilitas tus datos Debes facilitar los datos que pide este documento. Estos datos son necesarios para gestionar esta autorización. Si no facilitas estos datos, la UPM no puede realizar este trámite. Con quién puede compartir la UPM tus datos La UPM puede comunicar tu nombre y apellidos a las personas que vean el vídeo o las imágenes. La UPM puede hacerlo para reconocer tu autoría. Si no quieres que la UPM muestre tu nombre y apellidos, puedes oponerte de forma expresa. Tus derechos Tú tienes derecho a: acceder a tus datos rectificar tus datos pedir la cancelación o la supresión de tus datos oponerte al uso de tus datos pedir que la UPM limite el uso de tus datos Puedes pedir más información sobre estos derechos al Delegado de Protección de Datos de la UPM. Si no quedas conforme con la respuesta, puedes presentar una reclamación ante la Agencia Española de Protección de Datos. Página web: https://www.aepd.es/index.html</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -598,21 +596,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (Gemini 3.1 Pro)
-Facil B1</t>
+          <t>GPT 5.4 Think</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (Gemini 3.1 Pro)
-Facil B1</t>
+          <t>GPT 5.4 Think</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AUTORIZACIÓN PARA EL USO DE IMÁGENES Y VÍDEOS Yo, con nombre, apellidos, DNI y correo electrónico, doy permiso a la Universidad Politécnica de Madrid. Permito que la Universidad use las imágenes o grabaciones donde yo participo. El título del trabajo es: Con Inclusens todas las opiniones cuentan. Este material pertenece al proyecto de innovación educativa Inclusens 2.0. La Universidad publicará este material en internet para informar sobre sus actividades. Los canales de difusión serán YouTube, las páginas web de la Universidad, X y LinkedIn. La Universidad no usará estas imágenes para ganar dinero. Condiciones del permiso: Primero. La Universidad escribirá mi nombre para reconocer que soy el autor del material. Segundo. La Universidad puede usar el vídeo completo o solo una parte. Tercero. Yo aseguro que las imágenes cumplen las leyes de propiedad intelectual y de protección de datos. Por tanto, la Universidad no es responsable si hay problemas legales con el contenido. Cuarto. Este permiso no tiene límite de tiempo ni de lugar. Además, yo también puedo usar mis imágenes en otros sitios si quiero. Información sobre sus datos personales: La Universidad Politécnica de Madrid es la responsable de cuidar sus datos. Usamos su nombre y correo para gestionar esta autorización. Guardaremos sus datos de forma indefinida, a menos que usted pida borrarlos. La ley nos permite tratar sus datos porque usted firma este documento de forma voluntaria. Usted tiene derecho a ver sus datos y a pedir que los corrijamos si están mal. También puede pedir que los borremos. Para usar estos derechos, escriba un correo a proteccion.datos@upm.es. Si cree que no respetamos sus derechos, puede presentar una queja en la Agencia Española de Protección de Datos a través de su web. Firma y fecha.</t>
+          <t>Autorización para publicar imágenes o vídeos Datos de la persona que firma: Nombre y apellidos: DNI o pasaporte número: Correo electrónico: ¿Qué autorizas? Tú autorizas a la Universidad Politécnica de Madrid (en adelante, UPM) a publicar tus imágenes o vídeos. La UPM tiene el número de identificación fiscal Q-2818015-F. El vídeo o las imágenes tienen este título: Con Inclusens todas las opiniones cuentan Este vídeo o imágenes forman parte del proyecto: Aprendizaje-Servicio: Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores (INCLUSENS) 2.0 ¿Dónde se publicarán tus imágenes o vídeos? La UPM podrá publicar tus imágenes o vídeos en estos lugares: El canal oficial de la UPM en YouTube El portal de Aprendizaje-Servicio de la UPM: https://aprendizajeservicio.upm.es/ El portal de innovación educativa de la UPM: https://innovacioneducativa.upm.es La red social X: @IEducativa_UPM La red social LinkedIn: www.linkedin.com/in/aps.upm Esta publicación no tiene ningún fin comercial. Es decir, nadie ganará dinero con estas imágenes o vídeos. Condiciones que debes aceptar Al firmar este documento, aceptas estas condiciones: La UPM indicará de forma clara que tú eres el autor o autora del vídeo o las imágenes. La UPM podrá mostrar, compartir o publicar el vídeo o las imágenes, de forma completa o parcial, sin ganar dinero con ello. Tú afirmas que el vídeo o las imágenes respetan las leyes sobre: Protección de datos personales Derechos de imagen Propiedad intelectual o industrial Si alguien hace una reclamación relacionada con estos temas, la UPM no será responsable. Esta autorización no tiene límite de tiempo ni de lugar. Fecha y firma Tus datos personales La UPM usará tus datos personales para gestionar esta autorización. Me han informado de que puedo: Ver mis datos personales Corregir mis datos personales Pedir que borren mis datos personales Oponerme al uso de mis datos personales Limitar el uso de mis datos personales Puedo encontrar más información en el apartado siguiente. Información sobre la protección de tus datos ¿Quién es responsable de tus datos? La persona responsable de tus datos es: Universidad Politécnica de Madrid Oficina de Aprendizaje Servicio (ApS) Calle Ramiro de Maeztu, número 7, Madrid (28040) Puedes contactar con ellos: Por teléfono: 910 670 390 Por correo electrónico: oficina-aps@upm.es También puedes contactar con la persona responsable de la protección de datos: Por correo electrónico: proteccion.datos@upm.es ¿Para qué usan tus datos? La UPM usa tus datos para gestionar todo lo relacionado con esta autorización. ¿Cuánto tiempo guardarán tus datos? La UPM guardará tus datos de forma indefinida. Es decir, los guardará sin límite de tiempo, hasta que tú pidas que los borren. ¿Por qué pueden usar tus datos? La UPM puede usar tus datos porque: Tú has dado tu consentimiento para ello. Es necesario para cumplir con esta autorización. Esto está recogido en el Reglamento (UE) 2016/679, también llamado RGPD. El RGPD es la ley europea que protege tus datos personales. ¿Es obligatorio dar tus datos? Sí. Los datos que se piden son los necesarios para poder realizar esta autorización. Si no los das, no se podrá hacer la autorización. ¿Quién verá tus datos? Tu nombre y apellidos aparecerán en el vídeo o las imágenes para indicar que eres el autor o autora. Por eso, todas las personas que vean ese material conocerán tu nombre y apellidos. Si no quieres que esto ocurra, puedes indicarlo antes de firmar. ¿Cuáles son tus derechos? Tienes derecho a: Ver tus datos personales Corregir tus datos si son incorrectos Pedir que borren tus datos Oponerte a que usen tus datos Pedir que limiten el uso de tus datos Para ejercer estos derechos, puedes contactar con la persona responsable de la protección de datos en: proteccion.datos@upm.es Si sientes que no se respetan tus derechos, puedes presentar una queja ante la Agencia Española de Protección de Datos (AEPD). La AEPD es el organismo público que controla que las empresas e instituciones cumplan la ley de protección de datos. Puedes hacerlo en esta dirección de internet: https://www.aepd.es/index.html</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -627,21 +623,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (Gemini 3.1 Pro)
-Sencillo B2</t>
+          <t>Claude Sonnet 4.6</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (Gemini 3.1 Pro)
-Sencillo B2</t>
+          <t>Claude Sonnet 4.6</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AUTORIZACIÓN PARA USAR IMÁGENES Y VÍDEOS Datos de la persona que firma Nombre y apellidos: DNI o Pasaporte: Correo electrónico: Yo autorizo a la Universidad Politécnica de Madrid, también llamada UPM, a publicar mis imágenes o grabaciones. El título del trabajo es: CON INCLUSENS TODAS LAS OPINIONES CUENTAN. Este material forma parte del proyecto de innovación educativa INCLUSENS 2.0. Uso de las imágenes La UPM publicará este material en internet para mostrar sus actividades. La universidad no usará estas imágenes para obtener beneficios económicos. Los canales de difusión serán el canal de Youtube de la UPM, sus páginas web oficiales y sus redes sociales de X y LinkedIn. Condiciones del acuerdo Primero. La UPM mencionará mi nombre como autor en los vídeos o imágenes. Segundo. La universidad puede usar el contenido completo o solo una parte. Tercero. Yo aseguro que las imágenes cumplen la ley y respetan los derechos de otras personas. Por tanto, la UPM no es responsable de posibles problemas legales con el contenido. Cuarto. Este permiso no tiene límite de tiempo ni de lugar. Además, yo también puedo seguir usando mi material en otros sitios. Información sobre sus datos personales La UPM es la responsable de cuidar sus datos. El objetivo es gestionar este permiso de uso de imagen. La universidad guardará sus datos siempre, aunque usted puede pedir que los borren cuando quiera. Es necesario que facilite sus datos para poder tramitar esta autorización. Su nombre y apellidos aparecerán en el material para reconocer que usted es el autor. Si no quiere que su nombre sea público, debe avisar a la universidad. Sus derechos Usted tiene derecho a ver sus datos y a pedir que los cambien si son incorrectos. También puede pedir que dejen de usarlos o que los eliminen. Para usar estos derechos, puede escribir al correo proteccion.datos@upm.es. Si no está satisfecho, puede presentar una queja en la Agencia Española de Protección de Datos a través de su página web. Fecha y firma:</t>
+          <t>Permiso para usar fotos o vídeos Yo, (nombre completo de la persona) con DNI o Pasaporte número (número del documento) y con el correo electrónico (dirección de correo) doy permiso a la Universidad Politécnica de Madrid. A la Universidad se le llama UPM. Doy permiso para usar fotos o grabaciones en las que salgo. El título del trabajo es: CON INCLUSENS TODAS LAS OPINIONES CUENTAN. Este trabajo es parte del proyecto INCLUSENS 2.0. El proyecto busca crear herramientas inclusivas para personas con discapacidad cognitiva. La UPM puede publicar estas fotos o vídeos. Puede publicarlos en internet. No los usará para ganar dinero. Los publicará en estos lugares: - El canal oficial de Youtube de la UPM. - La página web de Aprendizaje-Servicio de la UPM. - La página web de innovación educativa de la UPM. - La red social X (antes Twitter) de la UPM. - La red social Linkedin de la UPM. Condiciones del permiso 1. La UPM dirá claramente que soy el autor o la autora de las fotos o vídeos. 2. La UPM puede copiar, repartir o mostrar los vídeos. Puede hacerlo de forma completa o en partes. No obtendrá ningún beneficio comercial. 3. Yo digo que el contenido de las fotos o vídeos respeta la ley. Respeto las leyes de protección de datos, de imagen y de propiedad intelectual. No haré reclamaciones a la Universidad por este uso. 4. Este permiso no es exclusivo. No tiene límite de tiempo. No tiene límite de lugar. Fecha y firma de la persona Información sobre el uso de mis datos personales Me han informado y doy mi consentimiento. La Universidad Politécnica de Madrid usará mis datos personales. La Oficina de Aprendizaje Servicio (ApS) es la responsable de usarlos. El objetivo es gestionar todo lo relacionado con este permiso. También me han informado de mis derechos. Puedo acceder a mis datos, corregirlos y pedir que los borren. Puedo hacer otras cosas con mis datos. Toda esta información está disponible al dorso de este documento. Más información sobre protección de datos ¿Quién usa mis datos? - Responsable: Universidad Politécnica de Madrid. Oficina de Aprendizaje Servicio (ApS). - Dirección: Calle Ramiro de Maeztu, 7. 28040 Madrid. - Teléfono: 9106 70390. - Correo electrónico: oficina-aps@upm.es. - Contacto del Delegado de Protección de Datos: proteccion.datos@upm.es. ¿Para qué usa mis datos? Usa mis datos para gestionar todo lo relacionado con este permiso. ¿Durante cuánto tiempo guarda mis datos? Guarda mis datos para siempre. Solo los borrará si yo lo pido. ¿Por qué puede usar mis datos? Puede usarlos por dos razones legales. 1. Porque es necesario para cumplir con este permiso. 2. Porque yo he dado mi consentimiento para ello. ¿Estoy obligado a dar estos datos? ¿Qué pasa si no los doy? Sí, debo dar estos datos. Son necesarios para hacer lo que pide este permiso. Si no los doy, no se podrá hacer. ¿A quién le dirá mis datos? Dirá mi nombre y apellidos a todas las personas que vean las fotos o vídeos. Lo hará para reconocer que soy el autor o la autora. No lo hará solo si yo digo expresamente que no quiero. ¿Qué derechos tengo sobre mis datos? Tengo estos derechos: - Acceder a mis datos. - Corregir mis datos si están mal. - Pedir que borren mis datos. - Oponeme a que los usen. - Pedir que limiten su uso. Puedo saber más sobre estos derechos. Puedo contactar con el Delegado de Protección de Datos de la UPM. Si no estoy contento con cómo se usan mis datos, puedo presentar una reclamación. Puedo hacerlo en la Agencia Española de Protección de Datos. Su página web es: https://www.aepd.es/index.html Glosas Protección de datos Es el derecho que tengo a controlar mi información personal. Por ejemplo, a decidir quién la usa y para qué. Datos personales Es cualquier información sobre mí. Por ejemplo, mi nombre, mi DNI o mi correo electrónico. Consentimiento Es decir que sí, estoy de acuerdo. Por ejemplo, dar permiso para que usen mis datos. Delegado de Protección de Datos Es la persona de una empresa que se encarga de que se respeten mis derechos sobre mis datos. Por ejemplo, a ella puedo dirigirme si tengo dudas o quejas.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -656,21 +650,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (Gemini 3.1 Pro)
-Sencillo B2.1</t>
+          <t>deepseek-v3.2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (Gemini 3.1 Pro)
-Sencillo B2.1</t>
+          <t>deepseek-v3.2</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Autorización para usar fotos y videos Una persona da permiso a la Universidad Politécnica de Madrid. La universidad se llama UPM. La UPM puede usar sus fotos y videos. El título del proyecto es: CON INCLUSENS TODAS LAS OPINIONES CUENTAN. La UPM puede publicar estas fotos y videos. Los puede publicar en internet. La UPM no gana dinero con esto. La UPM publicará el material en estos sitios: - Su canal de Youtube. - Su página web de Aprendizaje-Servicio. - Su página web de innovación educativa. - Sus redes sociales: X y Linkedin. Condiciones: 1. La UPM dirá el nombre del autor en el video o las fotos. 2. La UPM puede publicar el video entero o una parte. 3. La persona dice que el contenido cumple la ley. La UPM no tendrá problemas legales. 4. Este permiso no tiene fecha de fin. Este permiso es para todo el mundo. Fecha y firma. La UPM tratará sus datos personales. La UPM los usa para gestionar este permiso. Usted puede ver, cambiar o borrar sus datos. Puede pedir más información al dorso. Información sobre protección de datos ¿Quién usa sus datos? La Universidad Politécnica de Madrid. Su oficina de Aprendizaje-Servicio (ApS). Dirección: Calle Ramiro de Maeztu, 7, (28040 Madrid). Teléfono: 9106 70390. Email: oficina-aps@upm.es Email del Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué usa sus datos? Para gestionar la autorización que usted firma. ¿Por cuánto tiempo? Hasta que usted pida borrarlos. ¿Por qué puede la UPM usar sus datos? Porque usted da su permiso con esta firma. Porque es necesario para este trámite. ¿Tiene que dar sus datos? Sí. Si no los da, no puede hacer este trámite. ¿Quién verá sus datos? La UPM dirá su nombre en el video o las fotos. Todo el mundo que vea el material verá su nombre. Usted puede decir que no quiere esto. Tienes derechos sobre tus datos personales. Puedes pedir ver tus datos. Puedes pedir cambiar tus datos. Puedes pedir borrar tus datos. Puedes decir que no uses sus datos. Puedes pedir que usen menos tus datos. La ley dice que tienes estos derechos. Para saber más, habla con el Delegado de Protección de Datos. Esta persona trabaja en la UPM. Si no te ayudan, puedes quejarte. Puedes quejarte en la Agencia Española de Protección de Datos. Su página web es: https://www.aepd.es/index.html</t>
+          <t>AUTORIZACIÓN DE DIFUSIÓN DE IMAGEN/ VÍDEO don/ Doña, con Documento nacional de Identidad/ Pasaporte nº y con email( a efectos de tratamiento de los datos): , autoriza a la Universidad Politécnica de Madrid UPM ), a la difusión de las imágenes o de la grabación de su autoría / participación con título: CON INCLUSENS TODAS LAS OPINIONES CUENTAN en el Proyecto Aprendizaje-Servicio Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores( INCLUSENS) 2.0. Madrid es CIF Q-2818015-F( en adelante. CIF es el Código de Identificación Fiscal. Se prevé la posible difusión de este material audiovisual, incluido Internet que excluye su uso comercial. Internet es con sujeción a la finalidad del tratamiento descrita. Los canales utilizados serán: el canal oficial de Youtube de la UPM, el portal de ApS-UPM( https://aprendizajeservicio.upm.es/), de innovación educativa ( https://innovacioneducativa.upm.es) y en la red social de 10(@ IEducativa_UPM) y Linkedin( www.linkedin.com/in/aps.upm) Se asumen las siguientes condiciones: 1. La UPM hará un reconocimiento expreso de la autoría del firmante en el video / imágenes producidos. 2. La UPM podrá reproducir, distribuir o comunicar la grabación( incluido internet), de forma íntegra o parcial, sin obtener beneficio comercial alguno. 3. El firmante declara que los contenidos de la grabación/ imágenes observan: - la normativa vigente en materia de protección de datos de carácter personal, - derechos de imagen, - propiedad intelectual o - industrial, y exime a la Universidad de cualquier reclamación. 4. La presente autorización se realiza de forma no exclusiva, sin límite temporal o territorial. Fecha y firma He sido informado y consiento en que mis datos personales sean tratados por la Universidad Politécnica de Madrid responsable de este tratamiento, con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. Madrid es Oficina de Aprendizaje Servicio( ApS ). También se me ha informado de que puedo acceder, rectificar y suprimir los datos, y ejercer otros derechos, en los términos que se indican en la información adicional, disponible al dorso. INFORMACIÓN ADICIONALSOBRE PROTECCIÓN DE DATOS ¿ Quién es el responsable del tratamiento de sus datos? Universidad Politécnica de Madrid ( Oficina de Aprendizaje Servicio( ApS) Calle Ramiro de Maeztu( más de 28 mil Madrid) Tlf: más de 9 mil más de 70 mil; correo electrónico: oficina-aps @ upm.es Contacto Delegado de Protección de Datos: proteccion.datos@ upm.es ¿ Con qué finalidad se tratan sus datos personales? Sus datos personales de tratan con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. Maeztu es 7.¿Por cuánto tiempo conservaremos sus datos? Los datos personales se mantendrán en el sistema de forma indefinida en tanto el interesado no solicite su supresión. ¿ Cuál es la legitimación para el tratamiento de sus datos? Las bases legales que legitiman el tratamiento son las recogidas en el Reglamento( UE) 2016/679: Artículo RGPD: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para 1 o varios fines específicos. ¿ Tiene Ud. la obligación de facilitar estos datos personales y cuáles son las consecuencias de no hacerlo? Los datos solicitados son los de manera estricta necesarios para llevar a cabo el tratamiento, motivo por el que no será posible realizarlo si no los facilita. ¿ A qué destinatarios se comunicarán sus datos? Está previsto el reconocimiento expreso de la autoría del firmante en el video/ imágenes producidos, motivo por el que se comunicaría su nombre y apellidos a todas aquellas personas que visualicen el material autorizado, salvo oposición expresa por su parte. ¿ Cuáles son sus derechos en relación con los datos facilitados? En relación a los datos facilitados tiene derecho a acceder, rectificar, solicitar la cancelación y supresión, y a oponerse o a limitar el tratamiento de los mismos, en los términos establecidos de manera legal. Puede obtener más información sobre el ejercicio de estos derechos contactando con el Delegado de Protección de Datos de la UPM. Asimismo, y en el supuesto de que no obtenga satisfacción en el ejercicio de sus derechos, podrá presentar una reclamación ante la Agencia Española de Protección de Datos: https://www.aepd.es/ index.html Palabras difíciles: Email: Correo electrónico. El correo electrónico es como enviar cartas, pero por internet.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -685,21 +677,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (deepseek-v3.2)
-Muy A2</t>
+          <t>SimpleText (ClearText)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (deepseek-v3.2)
-Muy A2</t>
+          <t>SimpleText (ClearText)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Autorización para usar imágenes y vídeos Yo, (nombre de la persona), con DNI o pasaporte número (número) y email (email), autorizo a la Universidad Politécnica de Madrid (UPM) a usar mis imágenes o vídeos. El título del proyecto es: CON INCLUSENS TODAS LAS OPINIONES CUENTAN. La UPM puede publicar este material en internet, pero no para ganar dinero. Lo publicará en su canal de YouTube, en su portal de Aprendizaje-Servicio (ApS-UPM) y en sus redes sociales (X y Linkedin). Condiciones: 1. La UPM dirá que el material es mío. 2. La UPM puede usar el material completo o partes, pero sin obtener beneficios comerciales. 3. Yo confirmo que el material cumple todas las leyes y que la UPM no tendrá problemas legales por mi culpa. 4. Esta autorización no es exclusiva y no tiene límite de tiempo ni de lugar. Fecha y firma He recibido información y doy mi consentimiento para que la UPM use mis datos. La UPM los usará para gestionar esta autorización. Sé que puedo acceder, cambiar o eliminar mis datos. Más información está al dorso. Información adicional sobre protección de datos ¿Quién es responsable de sus datos? Universidad Politécnica de Madrid (Oficina de Aprendizaje-Servicio). Dirección: Calle Ramiro de Maeztu, 7, 28040 Madrid. Teléfono: 910670390. Email: oficina-aps@upm.es Contacto del Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué usamos sus datos? Para gestionar todo lo relacionado con esta autorización. ¿Cuánto tiempo guardaremos sus datos? Se guardarán para siempre hasta que usted pida eliminarlos. ¿Por qué podemos usar sus datos? Porque es necesario para hacer este trámite y porque usted nos da su consentimiento. ¿Tengo que dar estos datos? Sí, son necesarios. Sin ellos, no podemos hacer el trámite. ¿A quién se comunicarán sus datos? Se dirá su nombre y apellidos a quien vea el material, a menos que usted se oponga expresamente. ¿Cuáles son sus derechos sobre sus datos personales? Usted tiene derecho a acceder, corregir y borrar sus datos. También puede oponerse o limitar su uso, según la ley. Para saber más sobre estos derechos, contacte al Delegado de Protección de Datos de la UPM. Si no solucionan su problema, puede presentar una queja. Debe hacerlo en la Agencia Española de Protección de Datos (AEPD): https://www.aepd.es/index.html</t>
+          <t>Autorización de difusión de imagen o vídeo. D. Dña. con DNI / Pasaportes número y con email. Autoriza a la Universidad de Madrid a difundir las imágenes o la grabación de la persona. Título: Con inclusión todas las opiniones cuentan. En el proyecto Aprendizaje-Servicios. Desarrollo de herramientas inclusivas. Para personas con discapacidad cognitivo en las pruebas sensorial de consumidores. Se prevé la difusión de este material de vídeo en: El canal oficial de Youtube. El portal de Aprendizaje-Servici de la Universidad de Madrid. En la red social de Twitter y Linkedin., La Universidad Politécnica de Madrid (UPM) quiere usar el video o las imágenes que le des. En el video o las fotos tienes que poner el nombre de la persona que lo ha hecho. La UPM podrá usar el video o la foto en internet o en cualquier otro sitio. La UPG no podrá vender el video o la imagen. La UMG no podrá reclamar a la persona que ha hecho el video o la fotografía. La UMP no podrá reclamar por los datos personales que hay en el video o la fotogrfía. La UPI no podrá reclamar si la persona no ha dado su permiso para usar el video o imagen. La autorización es para siempre y para cualquier lugar., He sido informado y acepto que mis datos personales se usen por la Universidad Politecnica de Madrid, oficina de Aprendizaje Servicio, responsable de este tratamiento. También me han informado de que puedo ver, cambiar y borrar mis datos, así como hacer otros derechos, en la información que está en la parte de atrás., La Universidad Politécnica de la Universidad Politécnica Madrid es la responsable de los datos de los estudiantes que participan en el proyecto de Aprendizaje Servicio. Puedes contactar con la Oficina de Aprendizaje Servicio en la calle Ramiro de Maezu número 7 de Madrid. El teléfono es 910 67 03 90 y el correo electrónico es oficina-aps@ upm.es. Pueden contactar con el Delegado de Protección Datos en el correo electrónico proteccion.datos @upm.es., ¿Para qué utilizamos tus datos personales? Utilizamos tus datos personales para gestionar la autorización emitida y para cumplir con las obligaciones legales. ¿Cuánto tiempo conservaremos tus datos? Los conservaremos hasta que tú nos lo pidas., ¿Para qué voy a utilizar tus datos? Para poder darte el servicio que has pedido. Para poder darme cuenta de que eres una persona real y no un robot. Para poder contactarte si tienes alguna duda. ¿Puedes retirar tu consentimiento en cualquier momento? Sí. ¿Puede compartirse la información con otras entidades? No. ¿Cuánto tiempo voy a conservar tus datos? Hasta que dejes de utilizar el servicio. ¿Pues qué hago si no estoy de acuerdo con la política de privacidad? Puedes contactar con nosotros a través de este correo electrónico: ., ¿Tienes la obligación de facilitar tus datos personales y qué pasa si no lo haces? Los datos que piden son los necesarios para poder hacer el tratamiento. Si no los facilitas no podrán hacer el tratamiento., ¿A qué personas se comunicarán sus Datos? Se comunicarán sus datos a las personas que vean el video o imágenes que haya hecho. El firmante tendrá que reconocer que es el autor de las imágenes. Si el firmante no quiere que se sepa su nombre, no se comunicará., ¿Qué derechos tengo sobre los datos que doy? Tienes derecho a saber qué datos tienes, a cambiarlos, a pedir que los borren y a que no los usen. Puedes contactar con el Delegado/a de Protección de Datos para saber más sobre estos derechos. Si no estás satisfecho/a con la respuesta, puedes presentar una reclamación a la Agencia Española de protección de Datos: https//www.aepd.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -714,21 +704,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (deepseek-v3.2)
-Facil B1</t>
+          <t>Modelo_Qwen3.5_9B</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (deepseek-v3.2)
-Facil B1</t>
+          <t>Modelo_Qwen3.5_9B</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Autorización de uso de imagen y vídeo Yo, [Nombre], con DNI/Pasaporte número [Número] y email [Email], autorizo a la Universidad Politécnica de Madrid (UPM) a publicar imágenes o vídeos de mi participación en el proyecto: CON INCLUSENS TODAS LAS OPINIONES CUENTAN. Este material se usará en el proyecto INCLUSENS 2.0, que desarrolla herramientas para personas con discapacidad cognitiva. La UPM podrá difundir este material, sin fines comerciales, en sus canales oficiales: YouTube, su portal de Aprendizaje-Servicio (https://aprendizajeservicio.upm.es/), su web de innovación educativa (https://innovacioneducativa.upm.es) y en las redes sociales X (@IEducativa_UPM) y Linkedin (www.linkedin.com/in/aps.upm). Condiciones: 1. La UPM reconocerá mi autoría en el vídeo o las imágenes. 2. La UPM podrá reproducir, distribuir o comunicar la grabación, total o parcialmente, sin obtener beneficio comercial. 3. Yo declaro que el contenido cumple las normas de protección de datos, derechos de imagen y propiedad intelectual. Libero a la Universidad de cualquier reclamación. 4. Esta autorización no es exclusiva y no tiene límite de tiempo ni territorio. Fecha y firma He sido informado y doy mi consentimiento para que la Universidad Politécnica de Madrid (Oficina de Aprendizaje-Servicio) trate mis datos para gestionar esta autorización. Sé que puedo acceder, rectificar y suprimir mis datos, así como ejercer otros derechos, según la información adicional al dorso. Información adicional sobre protección de datos ¿Quién es responsable de sus datos? Universidad Politécnica de Madrid (Oficina de Aprendizaje-Servicio). Dirección: Calle Ramiro de Maeztu, 7, 28040 Madrid. Teléfono: 910670390; Email: oficina-aps@upm.es. Delegado de Protección de Datos: proteccion.datos@upm.es. ¿Para qué usamos sus datos? Para gestionar todos los aspectos de la autorización que ha firmado. ¿Cuánto tiempo conservamos sus datos? Se conservarán indefinidamente hasta que usted solicite su eliminación. ¿Por qué podemos tratar sus datos? Porque es necesario para ejecutar este acuerdo (artículo 6.1.b del Reglamento UE 2016/679) y porque usted nos ha dado su consentimiento (artículo 6.1.a). ¿Debe facilitar estos datos? Sí, son necesarios para realizar el trámite. No podemos hacerlo si no los facilita. ¿Se comunicarán sus datos a otras personas? Sí, se comunicará su nombre y apellidos a quienes vean el material para reconocer su autoría, a menos que usted se oponga expresamente. ¿Cuáles son sus derechos sobre sus datos personales? Usted tiene derecho a acceder, corregir, eliminar y oponerse al uso de sus datos, según la ley. Para más información, contacte con el Delegado de Protección de Datos de la UPM. Si no solucionan su problema, puede presentar una reclamación en la Agencia Española de Protección de Datos: https://www.aepd.es/index.html</t>
+          <t>Autorización para usar imágenes y vídeos Yo me llamo: Mi DNI o pasaporte es: Mi correo electrónico es: Yo autorizo a la Universidad Politécnica de Madrid (UPM) a usar y difundir las imágenes o vídeos en los que participo o que he creado. Título del material: CON INCLUSENS TODAS LAS OPINIONES CUENTAN Este material forma parte del proyecto: INCLUSENS 2.0 Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores. ¿Dónde puede aparecer el vídeo o las imágenes? La UPM puede publicar este material en: El canal oficial de YouTube de la UPM. La página web de Aprendizaje-Servicio de la UPM. La página web de Innovación Educativa de la UPM. La red social X. La red social LinkedIn. Internet. La UPM no puede usar este material con fines comerciales. Condiciones de la autorización La UPM reconocerá que tú eres la persona autora o participante del vídeo o de las imágenes. La UPM puede copiar, compartir o publicar el vídeo o las imágenes. La UPM puede publicar el material completo o una parte. La UPM no obtendrá beneficios comerciales con este material. Tú declaras que el contenido cumple la ley sobre: Protección de datos personales. Derecho a la propia imagen. Propiedad intelectual. Propiedad industrial. Si aparece algún problema relacionado con estos contenidos, la responsabilidad no será de la UPM. Esta autorización no tiene fecha de finalización. Esta autorización es válida en cualquier lugar. Fecha y firma Fecha: Firma: Información sobre tus datos personales La UPM tratará tus datos personales para gestionar esta autorización. Tú aceptas este tratamiento al firmar el documento. ¿Quién utiliza tus datos? Universidad Politécnica de Madrid (UPM) Oficina de Aprendizaje Servicio (ApS) Dirección: Calle Ramiro de Maeztu, 7. 28040 Madrid. Teléfono: 910 670 390 Correo electrónico: oficina-aps@upm.es Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué se usan tus datos? Tus datos se usan para gestionar esta autorización. ¿Durante cuánto tiempo se guardan tus datos? La UPM guardará tus datos mientras tú no solicites su eliminación. ¿Por qué puede la UPM usar tus datos? La UPM puede usar tus datos porque: Tú has dado tu consentimiento. La autorización firmada es necesaria para realizar esta actividad. ¿Es obligatorio dar estos datos? Sí. Estos datos son necesarios para gestionar la autorización. Si no facilitas estos datos, la UPM no podrá realizar este trámite. ¿Quién puede conocer tus datos? Si tu nombre aparece como autor o autora del vídeo o de las imágenes, cualquier persona que vea el material podrá conocer tu nombre y apellidos. Tú puedes solicitar que no aparezcan. ¿Qué derechos tienes? Tú puedes: Consultar tus datos. Corregir tus datos. Solicitar la eliminación de tus datos. Oponerte al uso de tus datos. Solicitar que se limite el uso de tus datos. Para ejercer estos derechos puedes contactar con el Delegado de Protección de Datos de la UPM. Correo electrónico: proteccion.datos@upm.es Si no estás de acuerdo con la respuesta recibida, puedes presentar una reclamación ante la Agencia Española de Protección de Datos. Página web: https://www.aepd.es Resumen Tú autorizas a la UPM a usar y difundir imágenes o vídeos. La UPM puede publicarlos en Internet y en sus redes sociales. La UPM no puede usarlos con fines comerciales. Tus datos personales se usarán para gestionar esta autorización.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -743,201 +731,10 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>AdaptaTuTexto (deepseek-v3.2)
-Sencillo B2</t>
+          <t>Asistente Lectura Facilitada "Francisco Javier Alvarez Jimenez"</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
-        <is>
-          <t>AdaptaTuTexto (deepseek-v3.2)
-Sencillo B2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Permiso para usar fotos y vídeos Tus datos Nombre y apellidos: Número de DNI o Pasaporte: Correo electrónico: Qué autorizas Das permiso a la Universidad Politécnica de Madrid para usar tus fotos o tus vídeos. La Universidad también se llama UPM. UPM Es el nombre corto de la Universidad Politécnica de Madrid. Tus fotos y vídeos se usan para el proyecto llamado: Con Inclusens todas las opiniones cuentan. Este proyecto crea herramientas para ayudar a personas con dificultades para comprender. Dónde se verán tus fotos y vídeos La Universidad puede publicar las imágenes en estos sitios: En el canal de Youtube de la Universidad. En las páginas de internet de la Universidad sobre aprendizaje e innovación. En la red social X. En la red social Linkedin. Reglas de este permiso La Universidad pondrá tu nombre para decir que tú eres el autor. La Universidad puede usar el vídeo entero o solo una parte. Nadie ganará dinero con tus fotos o vídeos. Tú aseguras que las fotos y vídeos cumplen las leyes. Este permiso es para siempre y para todos los países. Tus derechos y tus datos Tus datos personales son necesarios para gestionar este permiso. Datos personales Es la información que sirve para saber quién eres. Por ejemplo, tu nombre, tu número de DNI o tu correo electrónico. Tus derechos son: Saber qué datos tiene la Universidad sobre ti. Cambiar tus datos si están mal. Pedir que borren tus datos. Pedir que dejen de usar tus datos. Si quieres usar estos derechos, escribe un correo a: proteccion.datos@upm.es Si no estás de acuerdo con cómo usan tus datos, puedes quejarte en la Agencia Española de Protección de Datos. Firma Tú das tu permiso cuando firmas este papel. Fecha: de de 20 Firma: Información sobre la protección de tus datos ¿Quién cuida tus datos? La Universidad Politécnica de Madrid cuida tus datos. Dirección: Calle Ramiro de Maeztu, número 7. Madrid. Teléfono: 91 06 70 390. Correo electrónico: oficina-aps@upm.es ¿Para qué usa la Universidad tus datos? La Universidad usa tus datos para organizar el permiso que has firmado. ¿Cuánto tiempo guarda la Universidad tus datos? La Universidad guarda tus datos siempre, a menos que tú pidas que los borren. ¿Por qué puede la Universidad usar tus datos? La Universidad usa tus datos porque tú has dado tu permiso al firmar. También los usa para cumplir el acuerdo sobre tus fotos y vídeos. ¿Es obligatorio dar tus datos? Sí. Si no das tus datos, la Universidad no puede usar tus fotos o vídeos. ¿Quién más verá tus datos? Cualquier persona que vea los vídeos o fotos podrá ver tu nombre y apellidos. Tú puedes decir que no quieres que aparezca tu nombre.</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>AUTORIZACIÓN DE DIFUSIÓN DE IMAGEN/VÍDEO D./Dña. con DNI / Pasaporte nº y con email (a efectos de tratamiento de los datos): , autoriza a la Universidad Politécnica de Madrid, CIF Q-2818015-F (en adelante, UPM), a la difusión de las imágenes o de la grabación de su autoría/participación con título: CON INCLUSENS TODAS LAS OPINIONES CUENTAN en el Proyecto Aprendizaje-Servicio Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores (INCLUSENS) 2.0. Se prevé la posible difusión de este material audiovisual, incluido Internet, con sujeción a la finalidad del tratamiento descrita, que excluye su uso comercial. Los canales utilizados serán: el canal oficial de Youtube de la UPM, el portal de ApS-UPM (https://aprendizajeservicio.upm.es/), de innovación educativa (https://innovacioneducativa.upm.es) y en la red social de X (@IEducativa_UPM) y Linkedin (www.linkedin.com/in/aps.upm ) Se asumen las siguientes condiciones: 1. La UPM hará un reconocimiento expreso de la autoría del firmante en el video/imágenes producidos. 2. La UPM podrá reproducir, distribuir o comunicar la grabación (incluido internet), de forma íntegra o parcial, sin obtener beneficio comercial alguno. 3. El firmante declara que los contenidos de la grabación/imágenes observan la normativa vigente en materia de protección de datos de carácter personal, derechos de imagen, propiedad intelectual o industrial, y exime a la Universidad de cualquier reclamación. 4. La presente autorización se realiza de forma no exclusiva, sin límite temporal o territorial. Fecha y firma He sido informado y consiento en que mis datos personales sean tratados por la Universidad Politécnica de Madrid, Oficina de Aprendizaje Servicio (ApS), responsable de este tratamiento, con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. También se me ha informado de que puedo acceder, rectificar y suprimir los datos, así como ejercer otros derechos, en los términos que se indican en la información adicional, disponible al dorso. INFORMACIÓN ADICIONAL SOBRE PROTECCIÓN DE DATOS ¿Quién es el responsable del tratamiento de sus datos? Universidad Politécnica de Madrid (Oficina de Aprendizaje Servicio (ApS) Calle Ramiro de Maeztu, 7, (28040 Madrid) Tlf: 9106 70390; correo electrónico: oficina-aps@upm.es Contacto Delegado de Protección de Datos: proteccion.datos@upm.es ¿Con qué finalidad se tratan sus datos personales? Sus datos personales de tratan con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. ¿Por cuánto tiempo conservaremos sus datos? Los datos personales se mantendrán en el sistema de forma indefinida en tanto el interesado no solicite su supresión. ¿Cuál es la legitimación para el tratamiento de sus datos? Las bases legales que legitiman el tratamiento son las recogidas en el Reglamento (UE) 2016/679: Artículo RGPD: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Tiene Ud. la obligación de facilitar estos datos personales y cuáles son las consecuencias de no hacerlo? Los datos solicitados son los estrictamente necesarios para llevar a cabo el tratamiento, motivo por el que no será posible realizarlo si no los facilita. ¿A qué destinatarios se comunicarán sus datos? Está previsto el reconocimiento expreso de la autoría del firmante en el video/imágenes producidos, motivo por el que se comunicaría su nombre y apellidos a todas aquellas personas que visualicen el material autorizado, salvo oposición expresa por su parte. ¿Cuáles son sus derechos en relación con los datos facilitados? En relación a los datos facilitados tiene derecho a acceder, rectificar, solicitar la cancelación y supresión, y a oponerse o a limitar el tratamiento de los mismos, en los términos establecidos legalmente. Puede obtener más información sobre el ejercicio de estos derechos contactando con el Delegado de Protección de Datos de la UPM. Asimismo, y en el supuesto de que no obtenga satisfacción en el ejercicio de sus derechos, podrá presentar una reclamación ante la Agencia Española de Protección de Datos: https://www.aepd.es/index.html</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Permiso para usar mis fotos o vídeos Datos personales Nombre y apellidos: Número de Documento Nacional de Identidad o pasaporte: Correo electrónico: Doy permiso a la UPM o Universidad Politécnica de Madrid para usar y enseñar mis fotos o mis videos. Estas fotos o vídeos forman parte del Proyecto de la Oficina de Aprendizaje-Servicio llamado: ¿Para qué se usan mis fotos o vídeos? La UPM puede usar mis fotos o vídeos para contar y enseñar el proyecto. La UPM no gana dinero con la publicación de mis fotos o videos. Las fotos o vídeos pueden aparecer en los siguientes sitios de internet: el canal de YouTube de la UPM la web de Aprendizaje-Servicio: https://aprendizajeservicio.upm.es la web de Innovación Educativa: https://innovacioneducativa.upm.es el Linkedin de la UPM y en la red social X Reglas para usar mis fotos o videos 1. La UPM hará las fotos o los videos y pondrá mi nombre como participante. 2. La UPM puede copiar, compartir o enseñar las fotos y vídeos, completas o solo una parte. Todo esto puede realizarse en Internet. 3. La UPM dice que las fotos o los vídeos cumplen las leyes que protegen: los datos personales la imagen la propiedad intelectual La propiedad intelectual es que está protegido el uso de las fotos o videos. 4. La persona que firma este permiso no va a hacer ninguna reclamación a la UPM si hay algún problema con el contenido. 5. Este permiso no tiene límite en el tiempo y sirve para cualquier lugar. 6. Este permiso autoriza a la UPM a usar mis fotos o vídeos pero yo también puedo usarlas donde quiera. Firma y fecha: Fecha: Firma: En la siguiente página hay más información Más información Tengo la información sobre cómo se usarán mis datos personales. Doy mi permiso a la Universidad Politécnica de Madrid y a la Oficina de Aprendizaje-Servicio para usar y cuidar mis datos personales. La UPM usará mis datos para organizar y hacer todo lo relacionado con este permiso. La UPM también usará mis datos para cumplir este permiso. Sé que tengo derechos sobre mis datos y puedo: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo usar estos derechos según lo que se explica en la información que hay en la siguiente página. Más información sobre mis datos personales ¿Quién guarda y cuida mis datos? Oficina de Aprendizaje Servicio de la Universidad Politécnica de Madrid. Calle Ramiro de Maeztu número 7 28040 Madrid. Teléfono: 910 670 390 Correo electrónico: oficina-aps@upm.es Contacto: Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué usan mis datos? Mis datos personales se usan con el fin de tramitar este permiso. ¿Durante cuánto tiempo se guardan mis datos? La UPM guardará mis datos hasta que yo pida que los borren. ¿Cuál es la ley para el uso y protección de mis datos? La ley está en el Reglamento 2016/679: Artículo Reglamento General Protección de Datos: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Es necesario dar mis datos? Sí. Porque si no das tus datos, la UPM no puede tramitar este permiso. ¿A quién se comunicarán tus datos? Tu nombre y tus apellidos serán comunicados a todas las personas que vean las fotos o videos, cuando no digas lo contrario. ¿Qué puedo hacer con los datos que he facilitado? Con los datos que he facilitado tengo estos derechos: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo poner una queja cuando no estoy de acuerdo en la Agencia Española de Protección de Datos: https://www.aepd.es</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Gemini 3.1 Pro</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Gemini 3.1 Pro</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Autorización para difundir imagen o vídeo Yo, D./Dña. con DNI o pasaporte número y con correo electrónico doy permiso a la Universidad Politécnica de Madrid, UPM, con CIF Q-2818015-F, para difundir imágenes o una grabación en la que participo o que he creado. Título del material Con Inclusens todas las opiniones cuentan Proyecto Aprendizaje-Servicio. Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores. INCLUSENS 2.0. Dónde puede difundir la UPM este material La UPM puede difundir este material en internet. La UPM puede usar estos canales: el canal oficial de YouTube de la UPM el portal de ApS-UPM: https://aprendizajeservicio.upm.es/ el portal de innovación educativa: https://innovacioneducativa.upm.es la red social X: @IEducativa_UPM LinkedIn: www.linkedin.com/in/aps.upm La UPM usa este material solo para la finalidad de este proyecto. La UPM no usa este material con fines comerciales. Condiciones de esta autorización La UPM reconoce de forma expresa tu autoría en el vídeo o en las imágenes. La UPM puede reproducir, distribuir y comunicar la grabación o las imágenes. Puede hacerlo de forma completa o en parte. Puede hacerlo también en internet. La UPM no obtiene beneficio comercial con esta difusión. Tú declaras que el contenido cumple la ley sobre protección de datos personales, derecho a la imagen y propiedad intelectual o industrial. Tú aceptas que, si otra persona presenta una reclamación por estos temas, la UPM no tendrá responsabilidad. Esta autorización no es exclusiva. Esto significa que tú puedes autorizar también a otras personas o entidades. Esta autorización no tiene fecha de fin. Esta autorización vale para cualquier lugar. Fecha y firma Fecha: Firma: Consentimiento para usar tus datos personales He recibido información sobre el uso de mis datos personales. Doy mi consentimiento para que la Universidad Politécnica de Madrid, a través de la Oficina de Aprendizaje Servicio, ApS, use mis datos personales para gestionar todo lo relacionado con esta autorización. Información sobre protección de datos Datos personales Son los datos que sirven para identificarte. Ejemplo: tu nombre, tu DNI o tu correo electrónico. Tratamiento de datos Es el uso de tus datos para una finalidad concreta. Ejemplo: usar tu correo para gestionar esta autorización. Quién usa tus datos La Universidad Politécnica de Madrid. Oficina de Aprendizaje Servicio, ApS. Dirección: Calle Ramiro de Maeztu, 7. 28040 Madrid. Teléfono: 910670390. Correo electrónico: oficina-aps@upm.es Contacto sobre protección de datos Delegado de Protección de Datos Es la persona o el servicio que te ayuda con dudas o problemas sobre el uso de tus datos. Correo electrónico: proteccion.datos@upm.es Para qué usa la UPM tus datos La UPM usa tus datos para gestionar todo lo relacionado con esta autorización. Durante cuánto tiempo guarda la UPM tus datos La UPM guarda tus datos sin fecha de fin. La UPM los guarda hasta que tú pidas su supresión. Por qué la UPM puede usar tus datos La UPM puede usar tus datos por 2 motivos: porque este tratamiento es necesario para gestionar esta autorización porque tú das tu consentimiento para usar tus datos con esta finalidad Si no facilitas tus datos Debes facilitar los datos que pide este documento. Estos datos son necesarios para gestionar esta autorización. Si no facilitas estos datos, la UPM no puede realizar este trámite. Con quién puede compartir la UPM tus datos La UPM puede comunicar tu nombre y apellidos a las personas que vean el vídeo o las imágenes. La UPM puede hacerlo para reconocer tu autoría. Si no quieres que la UPM muestre tu nombre y apellidos, puedes oponerte de forma expresa. Tus derechos Tú tienes derecho a: acceder a tus datos rectificar tus datos pedir la cancelación o la supresión de tus datos oponerte al uso de tus datos pedir que la UPM limite el uso de tus datos Puedes pedir más información sobre estos derechos al Delegado de Protección de Datos de la UPM. Si no quedas conforme con la respuesta, puedes presentar una reclamación ante la Agencia Española de Protección de Datos. Página web: https://www.aepd.es/index.html</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>AUTORIZACIÓN DE DIFUSIÓN DE IMAGEN/VÍDEO D./Dña. con DNI / Pasaporte nº y con email (a efectos de tratamiento de los datos): , autoriza a la Universidad Politécnica de Madrid, CIF Q-2818015-F (en adelante, UPM), a la difusión de las imágenes o de la grabación de su autoría/participación con título: CON INCLUSENS TODAS LAS OPINIONES CUENTAN en el Proyecto Aprendizaje-Servicio Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores (INCLUSENS) 2.0. Se prevé la posible difusión de este material audiovisual, incluido Internet, con sujeción a la finalidad del tratamiento descrita, que excluye su uso comercial. Los canales utilizados serán: el canal oficial de Youtube de la UPM, el portal de ApS-UPM (https://aprendizajeservicio.upm.es/), de innovación educativa (https://innovacioneducativa.upm.es) y en la red social de X (@IEducativa_UPM) y Linkedin (www.linkedin.com/in/aps.upm ) Se asumen las siguientes condiciones: 1. La UPM hará un reconocimiento expreso de la autoría del firmante en el video/imágenes producidos. 2. La UPM podrá reproducir, distribuir o comunicar la grabación (incluido internet), de forma íntegra o parcial, sin obtener beneficio comercial alguno. 3. El firmante declara que los contenidos de la grabación/imágenes observan la normativa vigente en materia de protección de datos de carácter personal, derechos de imagen, propiedad intelectual o industrial, y exime a la Universidad de cualquier reclamación. 4. La presente autorización se realiza de forma no exclusiva, sin límite temporal o territorial. Fecha y firma He sido informado y consiento en que mis datos personales sean tratados por la Universidad Politécnica de Madrid, Oficina de Aprendizaje Servicio (ApS), responsable de este tratamiento, con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. También se me ha informado de que puedo acceder, rectificar y suprimir los datos, así como ejercer otros derechos, en los términos que se indican en la información adicional, disponible al dorso. INFORMACIÓN ADICIONAL SOBRE PROTECCIÓN DE DATOS ¿Quién es el responsable del tratamiento de sus datos? Universidad Politécnica de Madrid (Oficina de Aprendizaje Servicio (ApS) Calle Ramiro de Maeztu, 7, (28040 Madrid) Tlf: 9106 70390; correo electrónico: oficina-aps@upm.es Contacto Delegado de Protección de Datos: proteccion.datos@upm.es ¿Con qué finalidad se tratan sus datos personales? Sus datos personales de tratan con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. ¿Por cuánto tiempo conservaremos sus datos? Los datos personales se mantendrán en el sistema de forma indefinida en tanto el interesado no solicite su supresión. ¿Cuál es la legitimación para el tratamiento de sus datos? Las bases legales que legitiman el tratamiento son las recogidas en el Reglamento (UE) 2016/679: Artículo RGPD: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Tiene Ud. la obligación de facilitar estos datos personales y cuáles son las consecuencias de no hacerlo? Los datos solicitados son los estrictamente necesarios para llevar a cabo el tratamiento, motivo por el que no será posible realizarlo si no los facilita. ¿A qué destinatarios se comunicarán sus datos? Está previsto el reconocimiento expreso de la autoría del firmante en el video/imágenes producidos, motivo por el que se comunicaría su nombre y apellidos a todas aquellas personas que visualicen el material autorizado, salvo oposición expresa por su parte. ¿Cuáles son sus derechos en relación con los datos facilitados? En relación a los datos facilitados tiene derecho a acceder, rectificar, solicitar la cancelación y supresión, y a oponerse o a limitar el tratamiento de los mismos, en los términos establecidos legalmente. Puede obtener más información sobre el ejercicio de estos derechos contactando con el Delegado de Protección de Datos de la UPM. Asimismo, y en el supuesto de que no obtenga satisfacción en el ejercicio de sus derechos, podrá presentar una reclamación ante la Agencia Española de Protección de Datos: https://www.aepd.es/index.html</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Permiso para usar mis fotos o vídeos Datos personales Nombre y apellidos: Número de Documento Nacional de Identidad o pasaporte: Correo electrónico: Doy permiso a la UPM o Universidad Politécnica de Madrid para usar y enseñar mis fotos o mis videos. Estas fotos o vídeos forman parte del Proyecto de la Oficina de Aprendizaje-Servicio llamado: ¿Para qué se usan mis fotos o vídeos? La UPM puede usar mis fotos o vídeos para contar y enseñar el proyecto. La UPM no gana dinero con la publicación de mis fotos o videos. Las fotos o vídeos pueden aparecer en los siguientes sitios de internet: el canal de YouTube de la UPM la web de Aprendizaje-Servicio: https://aprendizajeservicio.upm.es la web de Innovación Educativa: https://innovacioneducativa.upm.es el Linkedin de la UPM y en la red social X Reglas para usar mis fotos o videos 1. La UPM hará las fotos o los videos y pondrá mi nombre como participante. 2. La UPM puede copiar, compartir o enseñar las fotos y vídeos, completas o solo una parte. Todo esto puede realizarse en Internet. 3. La UPM dice que las fotos o los vídeos cumplen las leyes que protegen: los datos personales la imagen la propiedad intelectual La propiedad intelectual es que está protegido el uso de las fotos o videos. 4. La persona que firma este permiso no va a hacer ninguna reclamación a la UPM si hay algún problema con el contenido. 5. Este permiso no tiene límite en el tiempo y sirve para cualquier lugar. 6. Este permiso autoriza a la UPM a usar mis fotos o vídeos pero yo también puedo usarlas donde quiera. Firma y fecha: Fecha: Firma: En la siguiente página hay más información Más información Tengo la información sobre cómo se usarán mis datos personales. Doy mi permiso a la Universidad Politécnica de Madrid y a la Oficina de Aprendizaje-Servicio para usar y cuidar mis datos personales. La UPM usará mis datos para organizar y hacer todo lo relacionado con este permiso. La UPM también usará mis datos para cumplir este permiso. Sé que tengo derechos sobre mis datos y puedo: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo usar estos derechos según lo que se explica en la información que hay en la siguiente página. Más información sobre mis datos personales ¿Quién guarda y cuida mis datos? Oficina de Aprendizaje Servicio de la Universidad Politécnica de Madrid. Calle Ramiro de Maeztu número 7 28040 Madrid. Teléfono: 910 670 390 Correo electrónico: oficina-aps@upm.es Contacto: Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué usan mis datos? Mis datos personales se usan con el fin de tramitar este permiso. ¿Durante cuánto tiempo se guardan mis datos? La UPM guardará mis datos hasta que yo pida que los borren. ¿Cuál es la ley para el uso y protección de mis datos? La ley está en el Reglamento 2016/679: Artículo Reglamento General Protección de Datos: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Es necesario dar mis datos? Sí. Porque si no das tus datos, la UPM no puede tramitar este permiso. ¿A quién se comunicarán tus datos? Tu nombre y tus apellidos serán comunicados a todas las personas que vean las fotos o videos, cuando no digas lo contrario. ¿Qué puedo hacer con los datos que he facilitado? Con los datos que he facilitado tengo estos derechos: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo poner una queja cuando no estoy de acuerdo en la Agencia Española de Protección de Datos: https://www.aepd.es</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>GPT 5.4 Think</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>GPT 5.4 Think</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Autorización para publicar imágenes o vídeos Datos de la persona que firma: Nombre y apellidos: DNI o pasaporte número: Correo electrónico: ¿Qué autorizas? Tú autorizas a la Universidad Politécnica de Madrid (en adelante, UPM) a publicar tus imágenes o vídeos. La UPM tiene el número de identificación fiscal Q-2818015-F. El vídeo o las imágenes tienen este título: Con Inclusens todas las opiniones cuentan Este vídeo o imágenes forman parte del proyecto: Aprendizaje-Servicio: Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores (INCLUSENS) 2.0 ¿Dónde se publicarán tus imágenes o vídeos? La UPM podrá publicar tus imágenes o vídeos en estos lugares: El canal oficial de la UPM en YouTube El portal de Aprendizaje-Servicio de la UPM: https://aprendizajeservicio.upm.es/ El portal de innovación educativa de la UPM: https://innovacioneducativa.upm.es La red social X: @IEducativa_UPM La red social LinkedIn: www.linkedin.com/in/aps.upm Esta publicación no tiene ningún fin comercial. Es decir, nadie ganará dinero con estas imágenes o vídeos. Condiciones que debes aceptar Al firmar este documento, aceptas estas condiciones: La UPM indicará de forma clara que tú eres el autor o autora del vídeo o las imágenes. La UPM podrá mostrar, compartir o publicar el vídeo o las imágenes, de forma completa o parcial, sin ganar dinero con ello. Tú afirmas que el vídeo o las imágenes respetan las leyes sobre: Protección de datos personales Derechos de imagen Propiedad intelectual o industrial Si alguien hace una reclamación relacionada con estos temas, la UPM no será responsable. Esta autorización no tiene límite de tiempo ni de lugar. Fecha y firma Tus datos personales La UPM usará tus datos personales para gestionar esta autorización. Me han informado de que puedo: Ver mis datos personales Corregir mis datos personales Pedir que borren mis datos personales Oponerme al uso de mis datos personales Limitar el uso de mis datos personales Puedo encontrar más información en el apartado siguiente. Información sobre la protección de tus datos ¿Quién es responsable de tus datos? La persona responsable de tus datos es: Universidad Politécnica de Madrid Oficina de Aprendizaje Servicio (ApS) Calle Ramiro de Maeztu, número 7, Madrid (28040) Puedes contactar con ellos: Por teléfono: 910 670 390 Por correo electrónico: oficina-aps@upm.es También puedes contactar con la persona responsable de la protección de datos: Por correo electrónico: proteccion.datos@upm.es ¿Para qué usan tus datos? La UPM usa tus datos para gestionar todo lo relacionado con esta autorización. ¿Cuánto tiempo guardarán tus datos? La UPM guardará tus datos de forma indefinida. Es decir, los guardará sin límite de tiempo, hasta que tú pidas que los borren. ¿Por qué pueden usar tus datos? La UPM puede usar tus datos porque: Tú has dado tu consentimiento para ello. Es necesario para cumplir con esta autorización. Esto está recogido en el Reglamento (UE) 2016/679, también llamado RGPD. El RGPD es la ley europea que protege tus datos personales. ¿Es obligatorio dar tus datos? Sí. Los datos que se piden son los necesarios para poder realizar esta autorización. Si no los das, no se podrá hacer la autorización. ¿Quién verá tus datos? Tu nombre y apellidos aparecerán en el vídeo o las imágenes para indicar que eres el autor o autora. Por eso, todas las personas que vean ese material conocerán tu nombre y apellidos. Si no quieres que esto ocurra, puedes indicarlo antes de firmar. ¿Cuáles son tus derechos? Tienes derecho a: Ver tus datos personales Corregir tus datos si son incorrectos Pedir que borren tus datos Oponerte a que usen tus datos Pedir que limiten el uso de tus datos Para ejercer estos derechos, puedes contactar con la persona responsable de la protección de datos en: proteccion.datos@upm.es Si sientes que no se respetan tus derechos, puedes presentar una queja ante la Agencia Española de Protección de Datos (AEPD). La AEPD es el organismo público que controla que las empresas e instituciones cumplan la ley de protección de datos. Puedes hacerlo en esta dirección de internet: https://www.aepd.es/index.html</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>AUTORIZACIÓN DE DIFUSIÓN DE IMAGEN/VÍDEO D./Dña. con DNI / Pasaporte nº y con email (a efectos de tratamiento de los datos): , autoriza a la Universidad Politécnica de Madrid, CIF Q-2818015-F (en adelante, UPM), a la difusión de las imágenes o de la grabación de su autoría/participación con título: CON INCLUSENS TODAS LAS OPINIONES CUENTAN en el Proyecto Aprendizaje-Servicio Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores (INCLUSENS) 2.0. Se prevé la posible difusión de este material audiovisual, incluido Internet, con sujeción a la finalidad del tratamiento descrita, que excluye su uso comercial. Los canales utilizados serán: el canal oficial de Youtube de la UPM, el portal de ApS-UPM (https://aprendizajeservicio.upm.es/), de innovación educativa (https://innovacioneducativa.upm.es) y en la red social de X (@IEducativa_UPM) y Linkedin (www.linkedin.com/in/aps.upm ) Se asumen las siguientes condiciones: 1. La UPM hará un reconocimiento expreso de la autoría del firmante en el video/imágenes producidos. 2. La UPM podrá reproducir, distribuir o comunicar la grabación (incluido internet), de forma íntegra o parcial, sin obtener beneficio comercial alguno. 3. El firmante declara que los contenidos de la grabación/imágenes observan la normativa vigente en materia de protección de datos de carácter personal, derechos de imagen, propiedad intelectual o industrial, y exime a la Universidad de cualquier reclamación. 4. La presente autorización se realiza de forma no exclusiva, sin límite temporal o territorial. Fecha y firma He sido informado y consiento en que mis datos personales sean tratados por la Universidad Politécnica de Madrid, Oficina de Aprendizaje Servicio (ApS), responsable de este tratamiento, con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. También se me ha informado de que puedo acceder, rectificar y suprimir los datos, así como ejercer otros derechos, en los términos que se indican en la información adicional, disponible al dorso. INFORMACIÓN ADICIONAL SOBRE PROTECCIÓN DE DATOS ¿Quién es el responsable del tratamiento de sus datos? Universidad Politécnica de Madrid (Oficina de Aprendizaje Servicio (ApS) Calle Ramiro de Maeztu, 7, (28040 Madrid) Tlf: 9106 70390; correo electrónico: oficina-aps@upm.es Contacto Delegado de Protección de Datos: proteccion.datos@upm.es ¿Con qué finalidad se tratan sus datos personales? Sus datos personales de tratan con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. ¿Por cuánto tiempo conservaremos sus datos? Los datos personales se mantendrán en el sistema de forma indefinida en tanto el interesado no solicite su supresión. ¿Cuál es la legitimación para el tratamiento de sus datos? Las bases legales que legitiman el tratamiento son las recogidas en el Reglamento (UE) 2016/679: Artículo RGPD: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Tiene Ud. la obligación de facilitar estos datos personales y cuáles son las consecuencias de no hacerlo? Los datos solicitados son los estrictamente necesarios para llevar a cabo el tratamiento, motivo por el que no será posible realizarlo si no los facilita. ¿A qué destinatarios se comunicarán sus datos? Está previsto el reconocimiento expreso de la autoría del firmante en el video/imágenes producidos, motivo por el que se comunicaría su nombre y apellidos a todas aquellas personas que visualicen el material autorizado, salvo oposición expresa por su parte. ¿Cuáles son sus derechos en relación con los datos facilitados? En relación a los datos facilitados tiene derecho a acceder, rectificar, solicitar la cancelación y supresión, y a oponerse o a limitar el tratamiento de los mismos, en los términos establecidos legalmente. Puede obtener más información sobre el ejercicio de estos derechos contactando con el Delegado de Protección de Datos de la UPM. Asimismo, y en el supuesto de que no obtenga satisfacción en el ejercicio de sus derechos, podrá presentar una reclamación ante la Agencia Española de Protección de Datos: https://www.aepd.es/index.html</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Permiso para usar mis fotos o vídeos Datos personales Nombre y apellidos: Número de Documento Nacional de Identidad o pasaporte: Correo electrónico: Doy permiso a la UPM o Universidad Politécnica de Madrid para usar y enseñar mis fotos o mis videos. Estas fotos o vídeos forman parte del Proyecto de la Oficina de Aprendizaje-Servicio llamado: ¿Para qué se usan mis fotos o vídeos? La UPM puede usar mis fotos o vídeos para contar y enseñar el proyecto. La UPM no gana dinero con la publicación de mis fotos o videos. Las fotos o vídeos pueden aparecer en los siguientes sitios de internet: el canal de YouTube de la UPM la web de Aprendizaje-Servicio: https://aprendizajeservicio.upm.es la web de Innovación Educativa: https://innovacioneducativa.upm.es el Linkedin de la UPM y en la red social X Reglas para usar mis fotos o videos 1. La UPM hará las fotos o los videos y pondrá mi nombre como participante. 2. La UPM puede copiar, compartir o enseñar las fotos y vídeos, completas o solo una parte. Todo esto puede realizarse en Internet. 3. La UPM dice que las fotos o los vídeos cumplen las leyes que protegen: los datos personales la imagen la propiedad intelectual La propiedad intelectual es que está protegido el uso de las fotos o videos. 4. La persona que firma este permiso no va a hacer ninguna reclamación a la UPM si hay algún problema con el contenido. 5. Este permiso no tiene límite en el tiempo y sirve para cualquier lugar. 6. Este permiso autoriza a la UPM a usar mis fotos o vídeos pero yo también puedo usarlas donde quiera. Firma y fecha: Fecha: Firma: En la siguiente página hay más información Más información Tengo la información sobre cómo se usarán mis datos personales. Doy mi permiso a la Universidad Politécnica de Madrid y a la Oficina de Aprendizaje-Servicio para usar y cuidar mis datos personales. La UPM usará mis datos para organizar y hacer todo lo relacionado con este permiso. La UPM también usará mis datos para cumplir este permiso. Sé que tengo derechos sobre mis datos y puedo: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo usar estos derechos según lo que se explica en la información que hay en la siguiente página. Más información sobre mis datos personales ¿Quién guarda y cuida mis datos? Oficina de Aprendizaje Servicio de la Universidad Politécnica de Madrid. Calle Ramiro de Maeztu número 7 28040 Madrid. Teléfono: 910 670 390 Correo electrónico: oficina-aps@upm.es Contacto: Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué usan mis datos? Mis datos personales se usan con el fin de tramitar este permiso. ¿Durante cuánto tiempo se guardan mis datos? La UPM guardará mis datos hasta que yo pida que los borren. ¿Cuál es la ley para el uso y protección de mis datos? La ley está en el Reglamento 2016/679: Artículo Reglamento General Protección de Datos: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Es necesario dar mis datos? Sí. Porque si no das tus datos, la UPM no puede tramitar este permiso. ¿A quién se comunicarán tus datos? Tu nombre y tus apellidos serán comunicados a todas las personas que vean las fotos o videos, cuando no digas lo contrario. ¿Qué puedo hacer con los datos que he facilitado? Con los datos que he facilitado tengo estos derechos: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo poner una queja cuando no estoy de acuerdo en la Agencia Española de Protección de Datos: https://www.aepd.es</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Claude Sonnet 4.6</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Claude Sonnet 4.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Permiso para usar fotos o vídeos Yo, (nombre completo de la persona) con DNI o Pasaporte número (número del documento) y con el correo electrónico (dirección de correo) doy permiso a la Universidad Politécnica de Madrid. A la Universidad se le llama UPM. Doy permiso para usar fotos o grabaciones en las que salgo. El título del trabajo es: CON INCLUSENS TODAS LAS OPINIONES CUENTAN. Este trabajo es parte del proyecto INCLUSENS 2.0. El proyecto busca crear herramientas inclusivas para personas con discapacidad cognitiva. La UPM puede publicar estas fotos o vídeos. Puede publicarlos en internet. No los usará para ganar dinero. Los publicará en estos lugares: - El canal oficial de Youtube de la UPM. - La página web de Aprendizaje-Servicio de la UPM. - La página web de innovación educativa de la UPM. - La red social X (antes Twitter) de la UPM. - La red social Linkedin de la UPM. Condiciones del permiso 1. La UPM dirá claramente que soy el autor o la autora de las fotos o vídeos. 2. La UPM puede copiar, repartir o mostrar los vídeos. Puede hacerlo de forma completa o en partes. No obtendrá ningún beneficio comercial. 3. Yo digo que el contenido de las fotos o vídeos respeta la ley. Respeto las leyes de protección de datos, de imagen y de propiedad intelectual. No haré reclamaciones a la Universidad por este uso. 4. Este permiso no es exclusivo. No tiene límite de tiempo. No tiene límite de lugar. Fecha y firma de la persona Información sobre el uso de mis datos personales Me han informado y doy mi consentimiento. La Universidad Politécnica de Madrid usará mis datos personales. La Oficina de Aprendizaje Servicio (ApS) es la responsable de usarlos. El objetivo es gestionar todo lo relacionado con este permiso. También me han informado de mis derechos. Puedo acceder a mis datos, corregirlos y pedir que los borren. Puedo hacer otras cosas con mis datos. Toda esta información está disponible al dorso de este documento. Más información sobre protección de datos ¿Quién usa mis datos? - Responsable: Universidad Politécnica de Madrid. Oficina de Aprendizaje Servicio (ApS). - Dirección: Calle Ramiro de Maeztu, 7. 28040 Madrid. - Teléfono: 9106 70390. - Correo electrónico: oficina-aps@upm.es. - Contacto del Delegado de Protección de Datos: proteccion.datos@upm.es. ¿Para qué usa mis datos? Usa mis datos para gestionar todo lo relacionado con este permiso. ¿Durante cuánto tiempo guarda mis datos? Guarda mis datos para siempre. Solo los borrará si yo lo pido. ¿Por qué puede usar mis datos? Puede usarlos por dos razones legales. 1. Porque es necesario para cumplir con este permiso. 2. Porque yo he dado mi consentimiento para ello. ¿Estoy obligado a dar estos datos? ¿Qué pasa si no los doy? Sí, debo dar estos datos. Son necesarios para hacer lo que pide este permiso. Si no los doy, no se podrá hacer. ¿A quién le dirá mis datos? Dirá mi nombre y apellidos a todas las personas que vean las fotos o vídeos. Lo hará para reconocer que soy el autor o la autora. No lo hará solo si yo digo expresamente que no quiero. ¿Qué derechos tengo sobre mis datos? Tengo estos derechos: - Acceder a mis datos. - Corregir mis datos si están mal. - Pedir que borren mis datos. - Oponeme a que los usen. - Pedir que limiten su uso. Puedo saber más sobre estos derechos. Puedo contactar con el Delegado de Protección de Datos de la UPM. Si no estoy contento con cómo se usan mis datos, puedo presentar una reclamación. Puedo hacerlo en la Agencia Española de Protección de Datos. Su página web es: https://www.aepd.es/index.html Glosas Protección de datos Es el derecho que tengo a controlar mi información personal. Por ejemplo, a decidir quién la usa y para qué. Datos personales Es cualquier información sobre mí. Por ejemplo, mi nombre, mi DNI o mi correo electrónico. Consentimiento Es decir que sí, estoy de acuerdo. Por ejemplo, dar permiso para que usen mis datos. Delegado de Protección de Datos Es la persona de una empresa que se encarga de que se respeten mis derechos sobre mis datos. Por ejemplo, a ella puedo dirigirme si tengo dudas o quejas.</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>AUTORIZACIÓN DE DIFUSIÓN DE IMAGEN/VÍDEO D./Dña. con DNI / Pasaporte nº y con email (a efectos de tratamiento de los datos): , autoriza a la Universidad Politécnica de Madrid, CIF Q-2818015-F (en adelante, UPM), a la difusión de las imágenes o de la grabación de su autoría/participación con título: CON INCLUSENS TODAS LAS OPINIONES CUENTAN en el Proyecto Aprendizaje-Servicio Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores (INCLUSENS) 2.0. Se prevé la posible difusión de este material audiovisual, incluido Internet, con sujeción a la finalidad del tratamiento descrita, que excluye su uso comercial. Los canales utilizados serán: el canal oficial de Youtube de la UPM, el portal de ApS-UPM (https://aprendizajeservicio.upm.es/), de innovación educativa (https://innovacioneducativa.upm.es) y en la red social de X (@IEducativa_UPM) y Linkedin (www.linkedin.com/in/aps.upm ) Se asumen las siguientes condiciones: 1. La UPM hará un reconocimiento expreso de la autoría del firmante en el video/imágenes producidos. 2. La UPM podrá reproducir, distribuir o comunicar la grabación (incluido internet), de forma íntegra o parcial, sin obtener beneficio comercial alguno. 3. El firmante declara que los contenidos de la grabación/imágenes observan la normativa vigente en materia de protección de datos de carácter personal, derechos de imagen, propiedad intelectual o industrial, y exime a la Universidad de cualquier reclamación. 4. La presente autorización se realiza de forma no exclusiva, sin límite temporal o territorial. Fecha y firma He sido informado y consiento en que mis datos personales sean tratados por la Universidad Politécnica de Madrid, Oficina de Aprendizaje Servicio (ApS), responsable de este tratamiento, con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. También se me ha informado de que puedo acceder, rectificar y suprimir los datos, así como ejercer otros derechos, en los términos que se indican en la información adicional, disponible al dorso. INFORMACIÓN ADICIONAL SOBRE PROTECCIÓN DE DATOS ¿Quién es el responsable del tratamiento de sus datos? Universidad Politécnica de Madrid (Oficina de Aprendizaje Servicio (ApS) Calle Ramiro de Maeztu, 7, (28040 Madrid) Tlf: 9106 70390; correo electrónico: oficina-aps@upm.es Contacto Delegado de Protección de Datos: proteccion.datos@upm.es ¿Con qué finalidad se tratan sus datos personales? Sus datos personales de tratan con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. ¿Por cuánto tiempo conservaremos sus datos? Los datos personales se mantendrán en el sistema de forma indefinida en tanto el interesado no solicite su supresión. ¿Cuál es la legitimación para el tratamiento de sus datos? Las bases legales que legitiman el tratamiento son las recogidas en el Reglamento (UE) 2016/679: Artículo RGPD: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Tiene Ud. la obligación de facilitar estos datos personales y cuáles son las consecuencias de no hacerlo? Los datos solicitados son los estrictamente necesarios para llevar a cabo el tratamiento, motivo por el que no será posible realizarlo si no los facilita. ¿A qué destinatarios se comunicarán sus datos? Está previsto el reconocimiento expreso de la autoría del firmante en el video/imágenes producidos, motivo por el que se comunicaría su nombre y apellidos a todas aquellas personas que visualicen el material autorizado, salvo oposición expresa por su parte. ¿Cuáles son sus derechos en relación con los datos facilitados? En relación a los datos facilitados tiene derecho a acceder, rectificar, solicitar la cancelación y supresión, y a oponerse o a limitar el tratamiento de los mismos, en los términos establecidos legalmente. Puede obtener más información sobre el ejercicio de estos derechos contactando con el Delegado de Protección de Datos de la UPM. Asimismo, y en el supuesto de que no obtenga satisfacción en el ejercicio de sus derechos, podrá presentar una reclamación ante la Agencia Española de Protección de Datos: https://www.aepd.es/index.html</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Permiso para usar mis fotos o vídeos Datos personales Nombre y apellidos: Número de Documento Nacional de Identidad o pasaporte: Correo electrónico: Doy permiso a la UPM o Universidad Politécnica de Madrid para usar y enseñar mis fotos o mis videos. Estas fotos o vídeos forman parte del Proyecto de la Oficina de Aprendizaje-Servicio llamado: ¿Para qué se usan mis fotos o vídeos? La UPM puede usar mis fotos o vídeos para contar y enseñar el proyecto. La UPM no gana dinero con la publicación de mis fotos o videos. Las fotos o vídeos pueden aparecer en los siguientes sitios de internet: el canal de YouTube de la UPM la web de Aprendizaje-Servicio: https://aprendizajeservicio.upm.es la web de Innovación Educativa: https://innovacioneducativa.upm.es el Linkedin de la UPM y en la red social X Reglas para usar mis fotos o videos 1. La UPM hará las fotos o los videos y pondrá mi nombre como participante. 2. La UPM puede copiar, compartir o enseñar las fotos y vídeos, completas o solo una parte. Todo esto puede realizarse en Internet. 3. La UPM dice que las fotos o los vídeos cumplen las leyes que protegen: los datos personales la imagen la propiedad intelectual La propiedad intelectual es que está protegido el uso de las fotos o videos. 4. La persona que firma este permiso no va a hacer ninguna reclamación a la UPM si hay algún problema con el contenido. 5. Este permiso no tiene límite en el tiempo y sirve para cualquier lugar. 6. Este permiso autoriza a la UPM a usar mis fotos o vídeos pero yo también puedo usarlas donde quiera. Firma y fecha: Fecha: Firma: En la siguiente página hay más información Más información Tengo la información sobre cómo se usarán mis datos personales. Doy mi permiso a la Universidad Politécnica de Madrid y a la Oficina de Aprendizaje-Servicio para usar y cuidar mis datos personales. La UPM usará mis datos para organizar y hacer todo lo relacionado con este permiso. La UPM también usará mis datos para cumplir este permiso. Sé que tengo derechos sobre mis datos y puedo: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo usar estos derechos según lo que se explica en la información que hay en la siguiente página. Más información sobre mis datos personales ¿Quién guarda y cuida mis datos? Oficina de Aprendizaje Servicio de la Universidad Politécnica de Madrid. Calle Ramiro de Maeztu número 7 28040 Madrid. Teléfono: 910 670 390 Correo electrónico: oficina-aps@upm.es Contacto: Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué usan mis datos? Mis datos personales se usan con el fin de tramitar este permiso. ¿Durante cuánto tiempo se guardan mis datos? La UPM guardará mis datos hasta que yo pida que los borren. ¿Cuál es la ley para el uso y protección de mis datos? La ley está en el Reglamento 2016/679: Artículo Reglamento General Protección de Datos: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Es necesario dar mis datos? Sí. Porque si no das tus datos, la UPM no puede tramitar este permiso. ¿A quién se comunicarán tus datos? Tu nombre y tus apellidos serán comunicados a todas las personas que vean las fotos o videos, cuando no digas lo contrario. ¿Qué puedo hacer con los datos que he facilitado? Con los datos que he facilitado tengo estos derechos: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo poner una queja cuando no estoy de acuerdo en la Agencia Española de Protección de Datos: https://www.aepd.es</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>deepseek-v3.2</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>deepseek-v3.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>AUTORIZACIÓN DE DIFUSIÓN DE IMAGEN/ VÍDEO don/ Doña, con Documento nacional de Identidad/ Pasaporte nº y con email( a efectos de tratamiento de los datos): , autoriza a la Universidad Politécnica de Madrid UPM ), a la difusión de las imágenes o de la grabación de su autoría / participación con título: CON INCLUSENS TODAS LAS OPINIONES CUENTAN en el Proyecto Aprendizaje-Servicio Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores( INCLUSENS) 2.0. Madrid es CIF Q-2818015-F( en adelante. CIF es el Código de Identificación Fiscal. Se prevé la posible difusión de este material audiovisual, incluido Internet que excluye su uso comercial. Internet es con sujeción a la finalidad del tratamiento descrita. Los canales utilizados serán: el canal oficial de Youtube de la UPM, el portal de ApS-UPM( https://aprendizajeservicio.upm.es/), de innovación educativa ( https://innovacioneducativa.upm.es) y en la red social de 10(@ IEducativa_UPM) y Linkedin( www.linkedin.com/in/aps.upm) Se asumen las siguientes condiciones: 1. La UPM hará un reconocimiento expreso de la autoría del firmante en el video / imágenes producidos. 2. La UPM podrá reproducir, distribuir o comunicar la grabación( incluido internet), de forma íntegra o parcial, sin obtener beneficio comercial alguno. 3. El firmante declara que los contenidos de la grabación/ imágenes observan: - la normativa vigente en materia de protección de datos de carácter personal, - derechos de imagen, - propiedad intelectual o - industrial, y exime a la Universidad de cualquier reclamación. 4. La presente autorización se realiza de forma no exclusiva, sin límite temporal o territorial. Fecha y firma He sido informado y consiento en que mis datos personales sean tratados por la Universidad Politécnica de Madrid responsable de este tratamiento, con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. Madrid es Oficina de Aprendizaje Servicio( ApS ). También se me ha informado de que puedo acceder, rectificar y suprimir los datos, y ejercer otros derechos, en los términos que se indican en la información adicional, disponible al dorso. INFORMACIÓN ADICIONALSOBRE PROTECCIÓN DE DATOS ¿ Quién es el responsable del tratamiento de sus datos? Universidad Politécnica de Madrid ( Oficina de Aprendizaje Servicio( ApS) Calle Ramiro de Maeztu( más de 28 mil Madrid) Tlf: más de 9 mil más de 70 mil; correo electrónico: oficina-aps @ upm.es Contacto Delegado de Protección de Datos: proteccion.datos@ upm.es ¿ Con qué finalidad se tratan sus datos personales? Sus datos personales de tratan con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. Maeztu es 7.¿Por cuánto tiempo conservaremos sus datos? Los datos personales se mantendrán en el sistema de forma indefinida en tanto el interesado no solicite su supresión. ¿ Cuál es la legitimación para el tratamiento de sus datos? Las bases legales que legitiman el tratamiento son las recogidas en el Reglamento( UE) 2016/679: Artículo RGPD: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para 1 o varios fines específicos. ¿ Tiene Ud. la obligación de facilitar estos datos personales y cuáles son las consecuencias de no hacerlo? Los datos solicitados son los de manera estricta necesarios para llevar a cabo el tratamiento, motivo por el que no será posible realizarlo si no los facilita. ¿ A qué destinatarios se comunicarán sus datos? Está previsto el reconocimiento expreso de la autoría del firmante en el video/ imágenes producidos, motivo por el que se comunicaría su nombre y apellidos a todas aquellas personas que visualicen el material autorizado, salvo oposición expresa por su parte. ¿ Cuáles son sus derechos en relación con los datos facilitados? En relación a los datos facilitados tiene derecho a acceder, rectificar, solicitar la cancelación y supresión, y a oponerse o a limitar el tratamiento de los mismos, en los términos establecidos de manera legal. Puede obtener más información sobre el ejercicio de estos derechos contactando con el Delegado de Protección de Datos de la UPM. Asimismo, y en el supuesto de que no obtenga satisfacción en el ejercicio de sus derechos, podrá presentar una reclamación ante la Agencia Española de Protección de Datos: https://www.aepd.es/ index.html Palabras difíciles: Email: Correo electrónico. El correo electrónico es como enviar cartas, pero por internet.</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>AUTORIZACIÓN DE DIFUSIÓN DE IMAGEN/VÍDEO D./Dña. con DNI / Pasaporte nº y con email (a efectos de tratamiento de los datos): , autoriza a la Universidad Politécnica de Madrid, CIF Q-2818015-F (en adelante, UPM), a la difusión de las imágenes o de la grabación de su autoría/participación con título: CON INCLUSENS TODAS LAS OPINIONES CUENTAN en el Proyecto Aprendizaje-Servicio Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores (INCLUSENS) 2.0. Se prevé la posible difusión de este material audiovisual, incluido Internet, con sujeción a la finalidad del tratamiento descrita, que excluye su uso comercial. Los canales utilizados serán: el canal oficial de Youtube de la UPM, el portal de ApS-UPM (https://aprendizajeservicio.upm.es/), de innovación educativa (https://innovacioneducativa.upm.es) y en la red social de X (@IEducativa_UPM) y Linkedin (www.linkedin.com/in/aps.upm ) Se asumen las siguientes condiciones: 1. La UPM hará un reconocimiento expreso de la autoría del firmante en el video/imágenes producidos. 2. La UPM podrá reproducir, distribuir o comunicar la grabación (incluido internet), de forma íntegra o parcial, sin obtener beneficio comercial alguno. 3. El firmante declara que los contenidos de la grabación/imágenes observan la normativa vigente en materia de protección de datos de carácter personal, derechos de imagen, propiedad intelectual o industrial, y exime a la Universidad de cualquier reclamación. 4. La presente autorización se realiza de forma no exclusiva, sin límite temporal o territorial. Fecha y firma He sido informado y consiento en que mis datos personales sean tratados por la Universidad Politécnica de Madrid, Oficina de Aprendizaje Servicio (ApS), responsable de este tratamiento, con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. También se me ha informado de que puedo acceder, rectificar y suprimir los datos, así como ejercer otros derechos, en los términos que se indican en la información adicional, disponible al dorso. INFORMACIÓN ADICIONAL SOBRE PROTECCIÓN DE DATOS ¿Quién es el responsable del tratamiento de sus datos? Universidad Politécnica de Madrid (Oficina de Aprendizaje Servicio (ApS) Calle Ramiro de Maeztu, 7, (28040 Madrid) Tlf: 9106 70390; correo electrónico: oficina-aps@upm.es Contacto Delegado de Protección de Datos: proteccion.datos@upm.es ¿Con qué finalidad se tratan sus datos personales? Sus datos personales de tratan con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. ¿Por cuánto tiempo conservaremos sus datos? Los datos personales se mantendrán en el sistema de forma indefinida en tanto el interesado no solicite su supresión. ¿Cuál es la legitimación para el tratamiento de sus datos? Las bases legales que legitiman el tratamiento son las recogidas en el Reglamento (UE) 2016/679: Artículo RGPD: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Tiene Ud. la obligación de facilitar estos datos personales y cuáles son las consecuencias de no hacerlo? Los datos solicitados son los estrictamente necesarios para llevar a cabo el tratamiento, motivo por el que no será posible realizarlo si no los facilita. ¿A qué destinatarios se comunicarán sus datos? Está previsto el reconocimiento expreso de la autoría del firmante en el video/imágenes producidos, motivo por el que se comunicaría su nombre y apellidos a todas aquellas personas que visualicen el material autorizado, salvo oposición expresa por su parte. ¿Cuáles son sus derechos en relación con los datos facilitados? En relación a los datos facilitados tiene derecho a acceder, rectificar, solicitar la cancelación y supresión, y a oponerse o a limitar el tratamiento de los mismos, en los términos establecidos legalmente. Puede obtener más información sobre el ejercicio de estos derechos contactando con el Delegado de Protección de Datos de la UPM. Asimismo, y en el supuesto de que no obtenga satisfacción en el ejercicio de sus derechos, podrá presentar una reclamación ante la Agencia Española de Protección de Datos: https://www.aepd.es/index.html</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Permiso para usar mis fotos o vídeos Datos personales Nombre y apellidos: Número de Documento Nacional de Identidad o pasaporte: Correo electrónico: Doy permiso a la UPM o Universidad Politécnica de Madrid para usar y enseñar mis fotos o mis videos. Estas fotos o vídeos forman parte del Proyecto de la Oficina de Aprendizaje-Servicio llamado: ¿Para qué se usan mis fotos o vídeos? La UPM puede usar mis fotos o vídeos para contar y enseñar el proyecto. La UPM no gana dinero con la publicación de mis fotos o videos. Las fotos o vídeos pueden aparecer en los siguientes sitios de internet: el canal de YouTube de la UPM la web de Aprendizaje-Servicio: https://aprendizajeservicio.upm.es la web de Innovación Educativa: https://innovacioneducativa.upm.es el Linkedin de la UPM y en la red social X Reglas para usar mis fotos o videos 1. La UPM hará las fotos o los videos y pondrá mi nombre como participante. 2. La UPM puede copiar, compartir o enseñar las fotos y vídeos, completas o solo una parte. Todo esto puede realizarse en Internet. 3. La UPM dice que las fotos o los vídeos cumplen las leyes que protegen: los datos personales la imagen la propiedad intelectual La propiedad intelectual es que está protegido el uso de las fotos o videos. 4. La persona que firma este permiso no va a hacer ninguna reclamación a la UPM si hay algún problema con el contenido. 5. Este permiso no tiene límite en el tiempo y sirve para cualquier lugar. 6. Este permiso autoriza a la UPM a usar mis fotos o vídeos pero yo también puedo usarlas donde quiera. Firma y fecha: Fecha: Firma: En la siguiente página hay más información Más información Tengo la información sobre cómo se usarán mis datos personales. Doy mi permiso a la Universidad Politécnica de Madrid y a la Oficina de Aprendizaje-Servicio para usar y cuidar mis datos personales. La UPM usará mis datos para organizar y hacer todo lo relacionado con este permiso. La UPM también usará mis datos para cumplir este permiso. Sé que tengo derechos sobre mis datos y puedo: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo usar estos derechos según lo que se explica en la información que hay en la siguiente página. Más información sobre mis datos personales ¿Quién guarda y cuida mis datos? Oficina de Aprendizaje Servicio de la Universidad Politécnica de Madrid. Calle Ramiro de Maeztu número 7 28040 Madrid. Teléfono: 910 670 390 Correo electrónico: oficina-aps@upm.es Contacto: Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué usan mis datos? Mis datos personales se usan con el fin de tramitar este permiso. ¿Durante cuánto tiempo se guardan mis datos? La UPM guardará mis datos hasta que yo pida que los borren. ¿Cuál es la ley para el uso y protección de mis datos? La ley está en el Reglamento 2016/679: Artículo Reglamento General Protección de Datos: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Es necesario dar mis datos? Sí. Porque si no das tus datos, la UPM no puede tramitar este permiso. ¿A quién se comunicarán tus datos? Tu nombre y tus apellidos serán comunicados a todas las personas que vean las fotos o videos, cuando no digas lo contrario. ¿Qué puedo hacer con los datos que he facilitado? Con los datos que he facilitado tengo estos derechos: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo poner una queja cuando no estoy de acuerdo en la Agencia Española de Protección de Datos: https://www.aepd.es</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>SimpleText (ClearText)</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>SimpleText (ClearText)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Autorización de difusión de imagen o vídeo. D. Dña. con DNI / Pasaportes número y con email. Autoriza a la Universidad de Madrid a difundir las imágenes o la grabación de la persona. Título: Con inclusión todas las opiniones cuentan. En el proyecto Aprendizaje-Servicios. Desarrollo de herramientas inclusivas. Para personas con discapacidad cognitivo en las pruebas sensorial de consumidores. Se prevé la difusión de este material de vídeo en: El canal oficial de Youtube. El portal de Aprendizaje-Servici de la Universidad de Madrid. En la red social de Twitter y Linkedin., La Universidad Politécnica de Madrid (UPM) quiere usar el video o las imágenes que le des. En el video o las fotos tienes que poner el nombre de la persona que lo ha hecho. La UPM podrá usar el video o la foto en internet o en cualquier otro sitio. La UPG no podrá vender el video o la imagen. La UMG no podrá reclamar a la persona que ha hecho el video o la fotografía. La UMP no podrá reclamar por los datos personales que hay en el video o la fotogrfía. La UPI no podrá reclamar si la persona no ha dado su permiso para usar el video o imagen. La autorización es para siempre y para cualquier lugar., He sido informado y acepto que mis datos personales se usen por la Universidad Politecnica de Madrid, oficina de Aprendizaje Servicio, responsable de este tratamiento. También me han informado de que puedo ver, cambiar y borrar mis datos, así como hacer otros derechos, en la información que está en la parte de atrás., La Universidad Politécnica de la Universidad Politécnica Madrid es la responsable de los datos de los estudiantes que participan en el proyecto de Aprendizaje Servicio. Puedes contactar con la Oficina de Aprendizaje Servicio en la calle Ramiro de Maezu número 7 de Madrid. El teléfono es 910 67 03 90 y el correo electrónico es oficina-aps@ upm.es. Pueden contactar con el Delegado de Protección Datos en el correo electrónico proteccion.datos @upm.es., ¿Para qué utilizamos tus datos personales? Utilizamos tus datos personales para gestionar la autorización emitida y para cumplir con las obligaciones legales. ¿Cuánto tiempo conservaremos tus datos? Los conservaremos hasta que tú nos lo pidas., ¿Para qué voy a utilizar tus datos? Para poder darte el servicio que has pedido. Para poder darme cuenta de que eres una persona real y no un robot. Para poder contactarte si tienes alguna duda. ¿Puedes retirar tu consentimiento en cualquier momento? Sí. ¿Puede compartirse la información con otras entidades? No. ¿Cuánto tiempo voy a conservar tus datos? Hasta que dejes de utilizar el servicio. ¿Pues qué hago si no estoy de acuerdo con la política de privacidad? Puedes contactar con nosotros a través de este correo electrónico: ., ¿Tienes la obligación de facilitar tus datos personales y qué pasa si no lo haces? Los datos que piden son los necesarios para poder hacer el tratamiento. Si no los facilitas no podrán hacer el tratamiento., ¿A qué personas se comunicarán sus Datos? Se comunicarán sus datos a las personas que vean el video o imágenes que haya hecho. El firmante tendrá que reconocer que es el autor de las imágenes. Si el firmante no quiere que se sepa su nombre, no se comunicará., ¿Qué derechos tengo sobre los datos que doy? Tienes derecho a saber qué datos tienes, a cambiarlos, a pedir que los borren y a que no los usen. Puedes contactar con el Delegado/a de Protección de Datos para saber más sobre estos derechos. Si no estás satisfecho/a con la respuesta, puedes presentar una reclamación a la Agencia Española de protección de Datos: https//www.aepd.</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>AUTORIZACIÓN DE DIFUSIÓN DE IMAGEN/VÍDEO D./Dña. con DNI / Pasaporte nº y con email (a efectos de tratamiento de los datos): , autoriza a la Universidad Politécnica de Madrid, CIF Q-2818015-F (en adelante, UPM), a la difusión de las imágenes o de la grabación de su autoría/participación con título: CON INCLUSENS TODAS LAS OPINIONES CUENTAN en el Proyecto Aprendizaje-Servicio Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores (INCLUSENS) 2.0. Se prevé la posible difusión de este material audiovisual, incluido Internet, con sujeción a la finalidad del tratamiento descrita, que excluye su uso comercial. Los canales utilizados serán: el canal oficial de Youtube de la UPM, el portal de ApS-UPM (https://aprendizajeservicio.upm.es/), de innovación educativa (https://innovacioneducativa.upm.es) y en la red social de X (@IEducativa_UPM) y Linkedin (www.linkedin.com/in/aps.upm ) Se asumen las siguientes condiciones: 1. La UPM hará un reconocimiento expreso de la autoría del firmante en el video/imágenes producidos. 2. La UPM podrá reproducir, distribuir o comunicar la grabación (incluido internet), de forma íntegra o parcial, sin obtener beneficio comercial alguno. 3. El firmante declara que los contenidos de la grabación/imágenes observan la normativa vigente en materia de protección de datos de carácter personal, derechos de imagen, propiedad intelectual o industrial, y exime a la Universidad de cualquier reclamación. 4. La presente autorización se realiza de forma no exclusiva, sin límite temporal o territorial. Fecha y firma He sido informado y consiento en que mis datos personales sean tratados por la Universidad Politécnica de Madrid, Oficina de Aprendizaje Servicio (ApS), responsable de este tratamiento, con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. También se me ha informado de que puedo acceder, rectificar y suprimir los datos, así como ejercer otros derechos, en los términos que se indican en la información adicional, disponible al dorso. INFORMACIÓN ADICIONAL SOBRE PROTECCIÓN DE DATOS ¿Quién es el responsable del tratamiento de sus datos? Universidad Politécnica de Madrid (Oficina de Aprendizaje Servicio (ApS) Calle Ramiro de Maeztu, 7, (28040 Madrid) Tlf: 9106 70390; correo electrónico: oficina-aps@upm.es Contacto Delegado de Protección de Datos: proteccion.datos@upm.es ¿Con qué finalidad se tratan sus datos personales? Sus datos personales de tratan con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. ¿Por cuánto tiempo conservaremos sus datos? Los datos personales se mantendrán en el sistema de forma indefinida en tanto el interesado no solicite su supresión. ¿Cuál es la legitimación para el tratamiento de sus datos? Las bases legales que legitiman el tratamiento son las recogidas en el Reglamento (UE) 2016/679: Artículo RGPD: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Tiene Ud. la obligación de facilitar estos datos personales y cuáles son las consecuencias de no hacerlo? Los datos solicitados son los estrictamente necesarios para llevar a cabo el tratamiento, motivo por el que no será posible realizarlo si no los facilita. ¿A qué destinatarios se comunicarán sus datos? Está previsto el reconocimiento expreso de la autoría del firmante en el video/imágenes producidos, motivo por el que se comunicaría su nombre y apellidos a todas aquellas personas que visualicen el material autorizado, salvo oposición expresa por su parte. ¿Cuáles son sus derechos en relación con los datos facilitados? En relación a los datos facilitados tiene derecho a acceder, rectificar, solicitar la cancelación y supresión, y a oponerse o a limitar el tratamiento de los mismos, en los términos establecidos legalmente. Puede obtener más información sobre el ejercicio de estos derechos contactando con el Delegado de Protección de Datos de la UPM. Asimismo, y en el supuesto de que no obtenga satisfacción en el ejercicio de sus derechos, podrá presentar una reclamación ante la Agencia Española de Protección de Datos: https://www.aepd.es/index.html</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Permiso para usar mis fotos o vídeos Datos personales Nombre y apellidos: Número de Documento Nacional de Identidad o pasaporte: Correo electrónico: Doy permiso a la UPM o Universidad Politécnica de Madrid para usar y enseñar mis fotos o mis videos. Estas fotos o vídeos forman parte del Proyecto de la Oficina de Aprendizaje-Servicio llamado: ¿Para qué se usan mis fotos o vídeos? La UPM puede usar mis fotos o vídeos para contar y enseñar el proyecto. La UPM no gana dinero con la publicación de mis fotos o videos. Las fotos o vídeos pueden aparecer en los siguientes sitios de internet: el canal de YouTube de la UPM la web de Aprendizaje-Servicio: https://aprendizajeservicio.upm.es la web de Innovación Educativa: https://innovacioneducativa.upm.es el Linkedin de la UPM y en la red social X Reglas para usar mis fotos o videos 1. La UPM hará las fotos o los videos y pondrá mi nombre como participante. 2. La UPM puede copiar, compartir o enseñar las fotos y vídeos, completas o solo una parte. Todo esto puede realizarse en Internet. 3. La UPM dice que las fotos o los vídeos cumplen las leyes que protegen: los datos personales la imagen la propiedad intelectual La propiedad intelectual es que está protegido el uso de las fotos o videos. 4. La persona que firma este permiso no va a hacer ninguna reclamación a la UPM si hay algún problema con el contenido. 5. Este permiso no tiene límite en el tiempo y sirve para cualquier lugar. 6. Este permiso autoriza a la UPM a usar mis fotos o vídeos pero yo también puedo usarlas donde quiera. Firma y fecha: Fecha: Firma: En la siguiente página hay más información Más información Tengo la información sobre cómo se usarán mis datos personales. Doy mi permiso a la Universidad Politécnica de Madrid y a la Oficina de Aprendizaje-Servicio para usar y cuidar mis datos personales. La UPM usará mis datos para organizar y hacer todo lo relacionado con este permiso. La UPM también usará mis datos para cumplir este permiso. Sé que tengo derechos sobre mis datos y puedo: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo usar estos derechos según lo que se explica en la información que hay en la siguiente página. Más información sobre mis datos personales ¿Quién guarda y cuida mis datos? Oficina de Aprendizaje Servicio de la Universidad Politécnica de Madrid. Calle Ramiro de Maeztu número 7 28040 Madrid. Teléfono: 910 670 390 Correo electrónico: oficina-aps@upm.es Contacto: Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué usan mis datos? Mis datos personales se usan con el fin de tramitar este permiso. ¿Durante cuánto tiempo se guardan mis datos? La UPM guardará mis datos hasta que yo pida que los borren. ¿Cuál es la ley para el uso y protección de mis datos? La ley está en el Reglamento 2016/679: Artículo Reglamento General Protección de Datos: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Es necesario dar mis datos? Sí. Porque si no das tus datos, la UPM no puede tramitar este permiso. ¿A quién se comunicarán tus datos? Tu nombre y tus apellidos serán comunicados a todas las personas que vean las fotos o videos, cuando no digas lo contrario. ¿Qué puedo hacer con los datos que he facilitado? Con los datos que he facilitado tengo estos derechos: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo poner una queja cuando no estoy de acuerdo en la Agencia Española de Protección de Datos: https://www.aepd.es</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Modelo_Qwen3.5_9B</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Modelo_Qwen3.5_9B</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Autorización para usar imágenes y vídeos Yo me llamo: Mi DNI o pasaporte es: Mi correo electrónico es: Yo autorizo a la Universidad Politécnica de Madrid (UPM) a usar y difundir las imágenes o vídeos en los que participo o que he creado. Título del material: CON INCLUSENS TODAS LAS OPINIONES CUENTAN Este material forma parte del proyecto: INCLUSENS 2.0 Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores. ¿Dónde puede aparecer el vídeo o las imágenes? La UPM puede publicar este material en: El canal oficial de YouTube de la UPM. La página web de Aprendizaje-Servicio de la UPM. La página web de Innovación Educativa de la UPM. La red social X. La red social LinkedIn. Internet. La UPM no puede usar este material con fines comerciales. Condiciones de la autorización La UPM reconocerá que tú eres la persona autora o participante del vídeo o de las imágenes. La UPM puede copiar, compartir o publicar el vídeo o las imágenes. La UPM puede publicar el material completo o una parte. La UPM no obtendrá beneficios comerciales con este material. Tú declaras que el contenido cumple la ley sobre: Protección de datos personales. Derecho a la propia imagen. Propiedad intelectual. Propiedad industrial. Si aparece algún problema relacionado con estos contenidos, la responsabilidad no será de la UPM. Esta autorización no tiene fecha de finalización. Esta autorización es válida en cualquier lugar. Fecha y firma Fecha: Firma: Información sobre tus datos personales La UPM tratará tus datos personales para gestionar esta autorización. Tú aceptas este tratamiento al firmar el documento. ¿Quién utiliza tus datos? Universidad Politécnica de Madrid (UPM) Oficina de Aprendizaje Servicio (ApS) Dirección: Calle Ramiro de Maeztu, 7. 28040 Madrid. Teléfono: 910 670 390 Correo electrónico: oficina-aps@upm.es Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué se usan tus datos? Tus datos se usan para gestionar esta autorización. ¿Durante cuánto tiempo se guardan tus datos? La UPM guardará tus datos mientras tú no solicites su eliminación. ¿Por qué puede la UPM usar tus datos? La UPM puede usar tus datos porque: Tú has dado tu consentimiento. La autorización firmada es necesaria para realizar esta actividad. ¿Es obligatorio dar estos datos? Sí. Estos datos son necesarios para gestionar la autorización. Si no facilitas estos datos, la UPM no podrá realizar este trámite. ¿Quién puede conocer tus datos? Si tu nombre aparece como autor o autora del vídeo o de las imágenes, cualquier persona que vea el material podrá conocer tu nombre y apellidos. Tú puedes solicitar que no aparezcan. ¿Qué derechos tienes? Tú puedes: Consultar tus datos. Corregir tus datos. Solicitar la eliminación de tus datos. Oponerte al uso de tus datos. Solicitar que se limite el uso de tus datos. Para ejercer estos derechos puedes contactar con el Delegado de Protección de Datos de la UPM. Correo electrónico: proteccion.datos@upm.es Si no estás de acuerdo con la respuesta recibida, puedes presentar una reclamación ante la Agencia Española de Protección de Datos. Página web: https://www.aepd.es Resumen Tú autorizas a la UPM a usar y difundir imágenes o vídeos. La UPM puede publicarlos en Internet y en sus redes sociales. La UPM no puede usarlos con fines comerciales. Tus datos personales se usarán para gestionar esta autorización.</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>AUTORIZACIÓN DE DIFUSIÓN DE IMAGEN/VÍDEO D./Dña. con DNI / Pasaporte nº y con email (a efectos de tratamiento de los datos): , autoriza a la Universidad Politécnica de Madrid, CIF Q-2818015-F (en adelante, UPM), a la difusión de las imágenes o de la grabación de su autoría/participación con título: CON INCLUSENS TODAS LAS OPINIONES CUENTAN en el Proyecto Aprendizaje-Servicio Desarrollo de herramientas inclusivas para personas con discapacidad cognitiva en las pruebas sensoriales de consumidores (INCLUSENS) 2.0. Se prevé la posible difusión de este material audiovisual, incluido Internet, con sujeción a la finalidad del tratamiento descrita, que excluye su uso comercial. Los canales utilizados serán: el canal oficial de Youtube de la UPM, el portal de ApS-UPM (https://aprendizajeservicio.upm.es/), de innovación educativa (https://innovacioneducativa.upm.es) y en la red social de X (@IEducativa_UPM) y Linkedin (www.linkedin.com/in/aps.upm ) Se asumen las siguientes condiciones: 1. La UPM hará un reconocimiento expreso de la autoría del firmante en el video/imágenes producidos. 2. La UPM podrá reproducir, distribuir o comunicar la grabación (incluido internet), de forma íntegra o parcial, sin obtener beneficio comercial alguno. 3. El firmante declara que los contenidos de la grabación/imágenes observan la normativa vigente en materia de protección de datos de carácter personal, derechos de imagen, propiedad intelectual o industrial, y exime a la Universidad de cualquier reclamación. 4. La presente autorización se realiza de forma no exclusiva, sin límite temporal o territorial. Fecha y firma He sido informado y consiento en que mis datos personales sean tratados por la Universidad Politécnica de Madrid, Oficina de Aprendizaje Servicio (ApS), responsable de este tratamiento, con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. También se me ha informado de que puedo acceder, rectificar y suprimir los datos, así como ejercer otros derechos, en los términos que se indican en la información adicional, disponible al dorso. INFORMACIÓN ADICIONAL SOBRE PROTECCIÓN DE DATOS ¿Quién es el responsable del tratamiento de sus datos? Universidad Politécnica de Madrid (Oficina de Aprendizaje Servicio (ApS) Calle Ramiro de Maeztu, 7, (28040 Madrid) Tlf: 9106 70390; correo electrónico: oficina-aps@upm.es Contacto Delegado de Protección de Datos: proteccion.datos@upm.es ¿Con qué finalidad se tratan sus datos personales? Sus datos personales de tratan con la finalidad de gestionar todos aquellos aspectos relacionados con la autorización emitida. ¿Por cuánto tiempo conservaremos sus datos? Los datos personales se mantendrán en el sistema de forma indefinida en tanto el interesado no solicite su supresión. ¿Cuál es la legitimación para el tratamiento de sus datos? Las bases legales que legitiman el tratamiento son las recogidas en el Reglamento (UE) 2016/679: Artículo RGPD: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Tiene Ud. la obligación de facilitar estos datos personales y cuáles son las consecuencias de no hacerlo? Los datos solicitados son los estrictamente necesarios para llevar a cabo el tratamiento, motivo por el que no será posible realizarlo si no los facilita. ¿A qué destinatarios se comunicarán sus datos? Está previsto el reconocimiento expreso de la autoría del firmante en el video/imágenes producidos, motivo por el que se comunicaría su nombre y apellidos a todas aquellas personas que visualicen el material autorizado, salvo oposición expresa por su parte. ¿Cuáles son sus derechos en relación con los datos facilitados? En relación a los datos facilitados tiene derecho a acceder, rectificar, solicitar la cancelación y supresión, y a oponerse o a limitar el tratamiento de los mismos, en los términos establecidos legalmente. Puede obtener más información sobre el ejercicio de estos derechos contactando con el Delegado de Protección de Datos de la UPM. Asimismo, y en el supuesto de que no obtenga satisfacción en el ejercicio de sus derechos, podrá presentar una reclamación ante la Agencia Española de Protección de Datos: https://www.aepd.es/index.html</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Permiso para usar mis fotos o vídeos Datos personales Nombre y apellidos: Número de Documento Nacional de Identidad o pasaporte: Correo electrónico: Doy permiso a la UPM o Universidad Politécnica de Madrid para usar y enseñar mis fotos o mis videos. Estas fotos o vídeos forman parte del Proyecto de la Oficina de Aprendizaje-Servicio llamado: ¿Para qué se usan mis fotos o vídeos? La UPM puede usar mis fotos o vídeos para contar y enseñar el proyecto. La UPM no gana dinero con la publicación de mis fotos o videos. Las fotos o vídeos pueden aparecer en los siguientes sitios de internet: el canal de YouTube de la UPM la web de Aprendizaje-Servicio: https://aprendizajeservicio.upm.es la web de Innovación Educativa: https://innovacioneducativa.upm.es el Linkedin de la UPM y en la red social X Reglas para usar mis fotos o videos 1. La UPM hará las fotos o los videos y pondrá mi nombre como participante. 2. La UPM puede copiar, compartir o enseñar las fotos y vídeos, completas o solo una parte. Todo esto puede realizarse en Internet. 3. La UPM dice que las fotos o los vídeos cumplen las leyes que protegen: los datos personales la imagen la propiedad intelectual La propiedad intelectual es que está protegido el uso de las fotos o videos. 4. La persona que firma este permiso no va a hacer ninguna reclamación a la UPM si hay algún problema con el contenido. 5. Este permiso no tiene límite en el tiempo y sirve para cualquier lugar. 6. Este permiso autoriza a la UPM a usar mis fotos o vídeos pero yo también puedo usarlas donde quiera. Firma y fecha: Fecha: Firma: En la siguiente página hay más información Más información Tengo la información sobre cómo se usarán mis datos personales. Doy mi permiso a la Universidad Politécnica de Madrid y a la Oficina de Aprendizaje-Servicio para usar y cuidar mis datos personales. La UPM usará mis datos para organizar y hacer todo lo relacionado con este permiso. La UPM también usará mis datos para cumplir este permiso. Sé que tengo derechos sobre mis datos y puedo: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo usar estos derechos según lo que se explica en la información que hay en la siguiente página. Más información sobre mis datos personales ¿Quién guarda y cuida mis datos? Oficina de Aprendizaje Servicio de la Universidad Politécnica de Madrid. Calle Ramiro de Maeztu número 7 28040 Madrid. Teléfono: 910 670 390 Correo electrónico: oficina-aps@upm.es Contacto: Delegado de Protección de Datos: proteccion.datos@upm.es ¿Para qué usan mis datos? Mis datos personales se usan con el fin de tramitar este permiso. ¿Durante cuánto tiempo se guardan mis datos? La UPM guardará mis datos hasta que yo pida que los borren. ¿Cuál es la ley para el uso y protección de mis datos? La ley está en el Reglamento 2016/679: Artículo Reglamento General Protección de Datos: Artículo 6.1.b) Tratamiento necesario para la ejecución de un contrato en el que el interesado es parte. Artículo 6.1.a) el interesado dio su consentimiento para el tratamiento de sus datos personales para uno o varios fines específicos. ¿Es necesario dar mis datos? Sí. Porque si no das tus datos, la UPM no puede tramitar este permiso. ¿A quién se comunicarán tus datos? Tu nombre y tus apellidos serán comunicados a todas las personas que vean las fotos o videos, cuando no digas lo contrario. ¿Qué puedo hacer con los datos que he facilitado? Con los datos que he facilitado tengo estos derechos: ver los datos que la UPM tiene sobre mí pedir que cambien los datos si hay algún error pedir que borren los datos pedir que los datos no se usen más Puedo poner una queja cuando no estoy de acuerdo en la Agencia Española de Protección de Datos: https://www.aepd.es</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Asistente Lectura Facilitada "Francisco Javier Alvarez Jimenez"</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
         <is>
           <t>Asistente Lectura Facilitada "Francisco Javier Alvarez Jimenez"</t>
         </is>

</xml_diff>